<commit_message>
Update latest CRM improvements, UI styling, and database sync
</commit_message>
<xml_diff>
--- a/data/F21_REAL_ESTATE_CRM.xlsx
+++ b/data/F21_REAL_ESTATE_CRM.xlsx
@@ -469,11 +469,6 @@
           <t>light</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>{"themeId":"UIv5","vars":{"--navy-primary":"#134E4A","--navy-dark":"#134E4A","--navy-light":"#5F7A78","--navy-hover":"#5F7A78","--navy-accent":"#2DD4BF","--c-secondary":"#5F7A78","--c-bg":"#F4F7F6","--c-card":"#FFFFFF","--c-on-accent":"#134E4A","--text-primary":"#1A1A1A","--text-muted":"#6B7280"},"primary":"#134E4A","accent":"#2DD4BF","text":"#1A1A1A"}</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>2026-07-10T11:09:20.692Z</t>
@@ -486,7 +481,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-21T14:13:47.068Z</t>
+          <t>2026-08-21T05:23:50.112Z</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -615,7 +610,7 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>2820000000</v>
+        <v>30000000</v>
       </c>
     </row>
     <row r="5">
@@ -675,7 +670,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>2820000000</v>
+        <v>30000000</v>
       </c>
     </row>
     <row r="6">
@@ -735,7 +730,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>2820000000</v>
+        <v>30000000</v>
       </c>
     </row>
     <row r="7">
@@ -795,7 +790,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>2820000000</v>
+        <v>30000000</v>
       </c>
     </row>
   </sheetData>
@@ -832,7 +827,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[{"dealType":"Rent","propertyId":4,"leadId":null,"buyerName":"Tenant 3","buyerPhone":"03007000003","agent":"agent2","dealAmount":11750000,"commissionPct":100,"commissionAmt":11750000,"agentSharePct":40,"agentShareAmt":4700000,"agentPaidAt":"2025-07-01T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2025-06-01T11:09:32.063Z","amount":11750000,"method":"Cash","ref":"","notes":"Commission = first month","receivedBy":"agent3"}],"status":"Completed","closedAt":"2025-06-02T11:09:32.063Z","cancellationReason":"","notes":"Tenancy ended after 13 months — unit re-listed","createdBy":"agent3","created":"2025-06-01T11:09:32.063Z","id":6,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Rent","propertyId":4,"leadId":null,"buyerName":"Tenant 3","buyerPhone":"03007000003","agent":"agent3","dealAmount":125000,"commissionPct":100,"commissionAmt":125000,"agentSharePct":40,"agentShareAmt":50000,"agentPaidAt":"2025-07-01T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2025-06-01T11:09:32.063Z","amount":125000,"method":"Cash","ref":"","notes":"Commission = first month","receivedBy":"agent3"}],"status":"Completed","closedAt":"2025-06-02T11:09:32.063Z","cancellationReason":"","notes":"Tenancy ended after 13 months — unit re-listed","createdBy":"agent3","created":"2025-06-01T11:09:32.063Z","id":6,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -844,7 +839,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[{"dealType":"Rent","propertyId":9,"leadId":null,"buyerName":"Tenant 2","buyerPhone":"03007000002","agent":"agent2","dealAmount":32900000,"commissionPct":100,"commissionAmt":32900000,"agentSharePct":40,"agentShareAmt":13160000,"agentPaidAt":"2026-05-17T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2026-05-02T11:09:32.063Z","amount":32900000,"method":"Bank Transfer","ref":"TT-5102","notes":"Commission = first month","receivedBy":"agent3"}],"status":"Completed","closedAt":"2026-05-02T11:09:32.063Z","cancellationReason":"","notes":"Shop let on a 12-month contract","createdBy":"agent3","created":"2026-05-01T11:09:32.063Z","id":5,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Rent","propertyId":9,"leadId":null,"buyerName":"Tenant 2","buyerPhone":"03007000002","agent":"agent3","dealAmount":350000,"commissionPct":100,"commissionAmt":350000,"agentSharePct":40,"agentShareAmt":140000,"agentPaidAt":"2026-05-17T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2026-05-02T11:09:32.063Z","amount":350000,"method":"Bank Transfer","ref":"TT-5102","notes":"Commission = first month","receivedBy":"agent3"}],"status":"Completed","closedAt":"2026-05-02T11:09:32.063Z","cancellationReason":"","notes":"Shop let on a 12-month contract","createdBy":"agent3","created":"2026-05-01T11:09:32.063Z","id":5,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -856,7 +851,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[{"dealType":"Rent","propertyId":19,"leadId":null,"buyerName":"Tenant 4","buyerPhone":"03007000004","agent":"agent1","dealAmount":6110000,"commissionPct":100,"commissionAmt":6110000,"agentSharePct":40,"agentShareAmt":2444000,"agentPaidAt":"2026-06-21T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2026-06-16T11:09:32.063Z","amount":6110000,"method":"Cash","ref":"","notes":"Commission = first month","receivedBy":"agent1"}],"status":"Completed","closedAt":"2026-06-16T11:09:32.063Z","cancellationReason":"","notes":"Furnished studio let","createdBy":"agent1","created":"2026-06-16T11:09:32.063Z","id":9,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Rent","propertyId":19,"leadId":null,"buyerName":"Tenant 4","buyerPhone":"03007000004","agent":"agent1","dealAmount":65000,"commissionPct":100,"commissionAmt":65000,"agentSharePct":40,"agentShareAmt":26000,"agentPaidAt":"2026-06-21T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2026-06-16T11:09:32.063Z","amount":65000,"method":"Cash","ref":"","notes":"Commission = first month","receivedBy":"agent1"}],"status":"Completed","closedAt":"2026-06-16T11:09:32.063Z","cancellationReason":"","notes":"Furnished studio let","createdBy":"agent1","created":"2026-06-16T11:09:32.063Z","id":9,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -868,7 +863,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[{"dealType":"Sale","propertyId":17,"leadId":null,"buyerName":"Buyer 4","buyerPhone":"03006000004","agent":"agent2","dealAmount":2726000000,"commissionPct":1,"commissionAmt":27260000,"agentSharePct":40,"agentShareAmt":10904000,"agentPaidAt":"2026-07-21T11:09:32.063Z","tokenAmount":94000000,"payments":[{"date":"2026-07-12T11:09:32.063Z","amount":94000000,"method":"Cash","ref":"","notes":"Token money","receivedBy":"agent3"},{"date":"2026-07-16T11:09:32.063Z","amount":2632000000,"method":"Bank Transfer","ref":"TT-7714","notes":"Balance on transfer","receivedBy":"agent3"}],"status":"Completed","closedAt":"2026-07-16T11:09:32.063Z","cancellationReason":"","notes":"","createdBy":"agent3","created":"2026-07-12T11:09:32.063Z","id":8,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Sale","propertyId":17,"leadId":null,"buyerName":"Buyer 4","buyerPhone":"03006000004","agent":"agent3","dealAmount":29000000,"commissionPct":1,"commissionAmt":290000,"agentSharePct":40,"agentShareAmt":116000,"agentPaidAt":"2026-07-21T11:09:32.063Z","tokenAmount":1000000,"payments":[{"date":"2026-07-12T11:09:32.063Z","amount":1000000,"method":"Cash","ref":"","notes":"Token money","receivedBy":"agent3"},{"date":"2026-07-16T11:09:32.063Z","amount":28000000,"method":"Bank Transfer","ref":"TT-7714","notes":"Balance on transfer","receivedBy":"agent3"}],"status":"Completed","closedAt":"2026-07-16T11:09:32.063Z","cancellationReason":"","notes":"","createdBy":"agent3","created":"2026-07-12T11:09:32.063Z","id":8,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -880,7 +875,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[{"dealType":"Sale","propertyId":11,"leadId":null,"buyerName":"Buyer 1","buyerPhone":"03006000001","agent":"agent2","dealAmount":10340000000,"commissionPct":1,"commissionAmt":103400000,"agentSharePct":40,"agentShareAmt":41360000,"agentPaidAt":"2026-08-21T06:08:54.585Z","tokenAmount":470000000,"payments":[{"date":"2026-07-20T11:09:32.063Z","amount":470000000,"method":"Bank Transfer","ref":"TT-3310","notes":"Token money","receivedBy":"agent2"},{"date":"2026-07-22T11:09:32.063Z","amount":9870000000,"method":"Bank Transfer","ref":"TT-3388","notes":"Balance on transfer","receivedBy":"agent2"}],"status":"Completed","closedAt":"2026-07-22T11:09:32.063Z","cancellationReason":"","notes":"Transfer done at registrar office","createdBy":"agent2","created":"2026-07-20T11:09:32.063Z","id":3,"updated":"2026-08-21T06:08:54.585Z"}]</t>
+          <t>[{"dealType":"Sale","propertyId":11,"leadId":null,"buyerName":"Buyer 1","buyerPhone":"03006000001","agent":"agent2","dealAmount":110000000,"commissionPct":1,"commissionAmt":1100000,"agentSharePct":40,"agentShareAmt":440000,"agentPaidAt":null,"tokenAmount":5000000,"payments":[{"date":"2026-07-20T11:09:32.063Z","amount":5000000,"method":"Bank Transfer","ref":"TT-3310","notes":"Token money","receivedBy":"agent2"},{"date":"2026-07-22T11:09:32.063Z","amount":105000000,"method":"Bank Transfer","ref":"TT-3388","notes":"Balance on transfer","receivedBy":"agent2"}],"status":"Completed","closedAt":"2026-07-22T11:09:32.063Z","cancellationReason":"","notes":"Transfer done at registrar office","createdBy":"agent2","created":"2026-07-20T11:09:32.063Z","id":3,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -892,7 +887,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[{"dealType":"Rent","propertyId":10,"leadId":null,"buyerName":"Tenant 1","buyerPhone":"03007000001","agent":"agent1","dealAmount":8930000,"commissionPct":100,"commissionAmt":8930000,"agentSharePct":40,"agentShareAmt":3572000,"agentPaidAt":"2026-07-27T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2026-07-24T11:09:32.063Z","amount":8930000,"method":"Cash","ref":"","notes":"Commission = first month","receivedBy":"agent1"}],"status":"Completed","closedAt":"2026-07-24T11:09:32.063Z","cancellationReason":"","notes":"","createdBy":"agent1","created":"2026-07-24T11:09:32.063Z","id":2,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Rent","propertyId":10,"leadId":null,"buyerName":"Tenant 1","buyerPhone":"03007000001","agent":"agent1","dealAmount":95000,"commissionPct":100,"commissionAmt":95000,"agentSharePct":40,"agentShareAmt":38000,"agentPaidAt":"2026-07-27T11:09:32.063Z","tokenAmount":0,"payments":[{"date":"2026-07-24T11:09:32.063Z","amount":95000,"method":"Cash","ref":"","notes":"Commission = first month","receivedBy":"agent1"}],"status":"Completed","closedAt":"2026-07-24T11:09:32.063Z","cancellationReason":"","notes":"","createdBy":"agent1","created":"2026-07-24T11:09:32.063Z","id":2,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -904,7 +899,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[{"dealType":"Sale","propertyId":3,"leadId":5,"buyerName":"Lead 5","buyerPhone":"03001000005","agent":"agent1","dealAmount":7520000000,"commissionPct":1,"commissionAmt":75200000,"agentSharePct":40,"agentShareAmt":30080000,"agentPaidAt":null,"tokenAmount":188000000,"payments":[{"date":"2026-07-25T11:09:32.063Z","amount":188000000,"method":"Bank Transfer","ref":"TT-4821","notes":"Token money","receivedBy":"agent1"}],"status":"Agreement","closedAt":null,"cancellationReason":"","notes":"Agreement signing this week","createdBy":"agent1","created":"2026-07-25T11:09:32.063Z","id":1,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Sale","propertyId":3,"leadId":5,"buyerName":"Lead 5","buyerPhone":"03001000005","agent":"agent1","dealAmount":80000000,"commissionPct":1,"commissionAmt":800000,"agentSharePct":40,"agentShareAmt":320000,"agentPaidAt":null,"tokenAmount":2000000,"payments":[{"date":"2026-07-25T11:09:32.063Z","amount":2000000,"method":"Bank Transfer","ref":"TT-4821","notes":"Token money","receivedBy":"agent1"}],"status":"Agreement","closedAt":null,"cancellationReason":"","notes":"Agreement signing this week","createdBy":"agent1","created":"2026-07-25T11:09:32.063Z","id":1,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -916,7 +911,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[{"dealType":"Rent","propertyId":6,"leadId":null,"buyerName":"Buyer 2","buyerPhone":"03006000002","agent":"agent2","dealAmount":17390000,"commissionPct":100,"commissionAmt":17390000,"agentSharePct":40,"agentShareAmt":6956000,"agentPaidAt":null,"tokenAmount":0,"payments":[],"status":"Cancelled","closedAt":null,"cancellationReason":"Tenant backed out before agreement signing","notes":"","createdBy":"agent3","created":"2026-07-30T11:09:32.063Z","id":4,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Rent","propertyId":6,"leadId":null,"buyerName":"Buyer 2","buyerPhone":"03006000002","agent":"agent3","dealAmount":185000,"commissionPct":100,"commissionAmt":185000,"agentSharePct":40,"agentShareAmt":74000,"agentPaidAt":null,"tokenAmount":0,"payments":[],"status":"Cancelled","closedAt":null,"cancellationReason":"Tenant backed out before agreement signing","notes":"","createdBy":"agent3","created":"2026-07-30T11:09:32.063Z","id":4,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -928,7 +923,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[{"dealType":"Sale","propertyId":8,"leadId":null,"buyerName":"Buyer 3","buyerPhone":"03006000003","agent":"agent2","dealAmount":893000000,"commissionPct":1,"commissionAmt":8930000,"agentSharePct":40,"agentShareAmt":3572000,"agentPaidAt":null,"tokenAmount":47000000,"payments":[{"date":"2026-08-03T11:09:32.063Z","amount":47000000,"method":"Cash","ref":"","notes":"Token money","receivedBy":"agent2"}],"status":"Token","closedAt":null,"cancellationReason":"","notes":"Balance on plot transfer at the society office","createdBy":"agent2","created":"2026-08-03T11:09:32.063Z","id":7,"updated":"2026-08-05T11:09:32.118Z"}]</t>
+          <t>[{"dealType":"Sale","propertyId":8,"leadId":null,"buyerName":"Buyer 3","buyerPhone":"03006000003","agent":"agent2","dealAmount":9500000,"commissionPct":1,"commissionAmt":95000,"agentSharePct":40,"agentShareAmt":38000,"agentPaidAt":null,"tokenAmount":500000,"payments":[{"date":"2026-08-03T11:09:32.063Z","amount":500000,"method":"Cash","ref":"","notes":"Token money","receivedBy":"agent2"}],"status":"Token","closedAt":null,"cancellationReason":"","notes":"Balance on plot transfer at the society office","createdBy":"agent2","created":"2026-08-03T11:09:32.063Z","id":7,"updated":"2026-08-05T11:09:32.118Z"}]</t>
         </is>
       </c>
     </row>
@@ -966,7 +961,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[{"propertyId":4,"dealId":6,"tenantName":"Tenant 3","tenantPhone":"03007000003","monthlyRent":12925000,"securityDeposit":23500000,"startDate":"2025-06-01","endDate":"2026-07-06","rentDueDay":5,"status":"Ended","rentLog":[{"month":"2025-06","amount":11750000,"paidAt":"2025-06-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2025-07","amount":11750000,"paidAt":"2025-07-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-08","amount":11750000,"paidAt":"2025-08-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-09","amount":11750000,"paidAt":"2025-09-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2025-10","amount":11750000,"paidAt":"2025-10-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-11","amount":11750000,"paidAt":"2025-11-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-12","amount":11750000,"paidAt":"2025-12-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2026-01","amount":11750000,"paidAt":"2026-01-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-02","amount":11750000,"paidAt":"2026-02-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-03","amount":11750000,"paidAt":"2026-03-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2026-04","amount":11750000,"paidAt":"2026-04-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-05","amount":11750000,"paidAt":"2026-05-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-06","amount":11750000,"paidAt":"2026-06-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"}],"renewals":[{"date":"2026-06-01T11:09:33.076Z","oldRent":125000,"newRent":137500,"newEndDate":"2027-06-01","notes":"Annual renewal — 10% increment","byUser":"manager1"}],"maintenance":[{"id":1,"date":"2026-01-17","issue":"Kitchen tap leakage","status":"Fixed","cost":423000,"fixedAt":"2026-01-19T11:09:33.078Z","addedBy":"agent3"}],"depositRefund":{"amount":21620000,"deductions":1880000,"notes":"Paint touch-up and one broken window pane","refundedAt":"2026-07-08T11:09:33.078Z"},"notes":"Tenant relocated to another city — unit re-listed","createdBy":"agent3","created":"2025-06-01T11:09:33.078Z","id":3,"updated":"2026-08-05T11:09:33.132Z"}]</t>
+          <t>[{"propertyId":4,"dealId":6,"tenantName":"Tenant 3","tenantPhone":"03007000003","monthlyRent":137500,"securityDeposit":250000,"startDate":"2025-06-01","endDate":"2026-07-06","rentDueDay":5,"status":"Ended","rentLog":[{"month":"2025-06","amount":125000,"paidAt":"2025-06-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2025-07","amount":125000,"paidAt":"2025-07-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-08","amount":125000,"paidAt":"2025-08-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-09","amount":125000,"paidAt":"2025-09-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2025-10","amount":125000,"paidAt":"2025-10-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-11","amount":125000,"paidAt":"2025-11-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2025-12","amount":125000,"paidAt":"2025-12-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2026-01","amount":125000,"paidAt":"2026-01-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-02","amount":125000,"paidAt":"2026-02-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-03","amount":125000,"paidAt":"2026-03-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2026-04","amount":125000,"paidAt":"2026-04-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-05","amount":125000,"paidAt":"2026-05-05T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-06","amount":125000,"paidAt":"2026-06-05T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"}],"renewals":[{"date":"2026-06-01T11:09:33.076Z","oldRent":125000,"newRent":137500,"newEndDate":"2027-06-01","notes":"Annual renewal — 10% increment","byUser":"manager1"}],"maintenance":[{"id":1,"date":"2026-01-17","issue":"Kitchen tap leakage","status":"Fixed","cost":4500,"fixedAt":"2026-01-19T11:09:33.078Z","addedBy":"agent3"}],"depositRefund":{"amount":230000,"deductions":20000,"notes":"Paint touch-up and one broken window pane","refundedAt":"2026-07-08T11:09:33.078Z"},"notes":"Tenant relocated to another city — unit re-listed","createdBy":"agent3","created":"2025-06-01T11:09:33.078Z","id":3,"updated":"2026-08-05T11:09:33.132Z"}]</t>
         </is>
       </c>
     </row>
@@ -978,7 +973,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[{"propertyId":9,"dealId":5,"tenantName":"Tenant 2","tenantPhone":"03007000002","monthlyRent":32900000,"securityDeposit":65800000,"startDate":"2026-05-02","endDate":"2027-05-02","rentDueDay":1,"status":"Active","rentLog":[{"month":"2026-05","amount":32900000,"paidAt":"2026-05-01T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2026-06","amount":32900000,"paidAt":"2026-06-01T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-07","amount":32900000,"paidAt":"2026-07-01T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-08","amount":32900000,"paidAt":"2026-08-01T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"}],"renewals":[],"maintenance":[],"depositRefund":null,"notes":"Commercial shop — 12-month contract","createdBy":"agent3","created":"2026-05-02T11:09:33.074Z","id":2,"updated":"2026-08-05T11:09:33.132Z"}]</t>
+          <t>[{"propertyId":9,"dealId":5,"tenantName":"Tenant 2","tenantPhone":"03007000002","monthlyRent":350000,"securityDeposit":700000,"startDate":"2026-05-02","endDate":"2027-05-02","rentDueDay":1,"status":"Active","rentLog":[{"month":"2026-05","amount":350000,"paidAt":"2026-05-01T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"},{"month":"2026-06","amount":350000,"paidAt":"2026-06-01T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-07","amount":350000,"paidAt":"2026-07-01T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent3"},{"month":"2026-08","amount":350000,"paidAt":"2026-08-01T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent3"}],"renewals":[],"maintenance":[],"depositRefund":null,"notes":"Commercial shop — 12-month contract","createdBy":"agent3","created":"2026-05-02T11:09:33.074Z","id":2,"updated":"2026-08-05T11:09:33.132Z"}]</t>
         </is>
       </c>
     </row>
@@ -990,7 +985,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[{"propertyId":19,"dealId":9,"tenantName":"Tenant 4","tenantPhone":"03007000004","monthlyRent":6110000,"securityDeposit":12220000,"startDate":"2026-06-16","endDate":"2027-06-16","rentDueDay":10,"status":"Active","rentLog":[{"month":"2026-06","amount":6110000,"paidAt":"2026-06-10T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent1"},{"month":"2026-07","amount":6110000,"paidAt":"2026-07-10T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent1"}],"renewals":[],"maintenance":[],"depositRefund":null,"notes":"Furnished studio","createdBy":"agent1","created":"2026-06-16T11:09:33.079Z","id":4,"updated":"2026-08-05T11:09:33.132Z"}]</t>
+          <t>[{"propertyId":19,"dealId":9,"tenantName":"Tenant 4","tenantPhone":"03007000004","monthlyRent":65000,"securityDeposit":130000,"startDate":"2026-06-16","endDate":"2027-06-16","rentDueDay":10,"status":"Active","rentLog":[{"month":"2026-06","amount":65000,"paidAt":"2026-06-10T19:00:00.000Z","method":"Bank Transfer","ref":"","receivedBy":"agent1"},{"month":"2026-07","amount":65000,"paidAt":"2026-07-10T19:00:00.000Z","method":"Cash","ref":"","receivedBy":"agent1"}],"renewals":[],"maintenance":[],"depositRefund":null,"notes":"Furnished studio","createdBy":"agent1","created":"2026-06-16T11:09:33.079Z","id":4,"updated":"2026-08-05T11:09:33.132Z"}]</t>
         </is>
       </c>
     </row>
@@ -1002,7 +997,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[{"propertyId":10,"dealId":2,"tenantName":"Tenant 1","tenantPhone":"03007000001","monthlyRent":8930000,"securityDeposit":17860000,"startDate":"2026-06-26","endDate":"2026-08-25","rentDueDay":5,"status":"Active","rentLog":[{"month":"2026-07","amount":8930000,"paidAt":"2026-07-01T11:09:33.071Z","method":"Cash","ref":"","receivedBy":"agent1"}],"renewals":[],"maintenance":[{"id":1,"date":"2026-07-30","issue":"AC service needed in master bedroom","status":"Open","cost":0,"fixedAt":null,"addedBy":"agent1"}],"depositRefund":null,"notes":"","createdBy":"agent1","created":"2026-06-26T11:09:33.072Z","id":1,"updated":"2026-08-05T11:09:33.132Z"}]</t>
+          <t>[{"propertyId":10,"dealId":2,"tenantName":"Tenant 1","tenantPhone":"03007000001","monthlyRent":95000,"securityDeposit":190000,"startDate":"2026-06-26","endDate":"2026-08-25","rentDueDay":5,"status":"Active","rentLog":[{"month":"2026-07","amount":95000,"paidAt":"2026-07-01T11:09:33.071Z","method":"Cash","ref":"","receivedBy":"agent1"}],"renewals":[],"maintenance":[{"id":1,"date":"2026-07-30","issue":"AC service needed in master bedroom","status":"Open","cost":0,"fixedAt":null,"addedBy":"agent1"}],"depositRefund":null,"notes":"","createdBy":"agent1","created":"2026-06-26T11:09:33.072Z","id":1,"updated":"2026-08-05T11:09:33.132Z"}]</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1095,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[{"user":"admin","action":"System Setup","details":"Demo data initialized","created":"2026-07-22T11:09:34.022Z","id":1,"updated":"2026-08-05T11:09:34.074Z"},{"user":"admin","action":"Property Added","details":"RS-LAH-1001 252,93 m² Modern House Phase 5","created":"2026-07-22T11:09:34.022Z","id":2,"updated":"2026-08-05T11:09:34.074Z"}]</t>
+          <t>[{"user":"admin","action":"System Setup","details":"Demo data initialized","created":"2026-07-22T11:09:34.022Z","id":1,"updated":"2026-08-05T11:09:34.074Z"},{"user":"admin","action":"Property Added","details":"RS-LAH-1001 10 Marla Modern House Phase 5","created":"2026-07-22T11:09:34.022Z","id":2,"updated":"2026-08-05T11:09:34.074Z"}]</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1179,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[{"id":21,"user":"admin","action":"Appointment Added","details":"#21","created":"2026-08-21T05:50:24.200Z","updated":"2026-08-21T05:50:24.200Z"},{"id":22,"user":"admin","action":"FollowUp Updated","details":"#16","created":"2026-08-21T10:01:30.588Z","updated":"2026-08-21T10:01:30.588Z"},{"id":23,"user":"admin","action":"Profile Image Uploaded","details":"Cập nhật ảnh đại diện: ChatGPT Image 12_48_54 10 thg 8, 2026.png","created":"2026-08-21T14:13:46.047Z","updated":"2026-08-21T14:13:46.047Z"},{"id":24,"user":"admin","action":"Agency Branding Updated","details":"Đổi nhận diện: NTH CRM","created":"2026-08-21T14:24:39.693Z","updated":"2026-08-21T14:24:39.693Z"},{"id":25,"user":"admin","action":"Propertie Added","details":"#21","created":"2026-08-21T14:39:15.248Z","updated":"2026-08-21T14:39:15.248Z"},{"id":26,"user":"admin","action":"Lead Added","details":"#21","created":"2026-08-21T14:39:16.208Z","updated":"2026-08-21T14:39:16.208Z"},{"id":27,"user":"admin","action":"Appointment Added","details":"#22","created":"2026-08-21T14:39:17.172Z","updated":"2026-08-21T14:39:17.172Z"},{"id":28,"user":"admin","action":"FollowUp Added","details":"#21","created":"2026-08-21T14:39:18.192Z","updated":"2026-08-21T14:39:18.192Z"},{"id":29,"user":"admin","action":"Propertie Deleted","details":"#21","created":"2026-08-21T14:39:19.155Z","updated":"2026-08-21T14:39:19.155Z"},{"id":30,"user":"admin","action":"Lead Deleted","details":"#21","created":"2026-08-21T14:39:22.302Z","updated":"2026-08-21T14:39:22.302Z"}]</t>
+          <t>[{"id":21,"user":"admin","action":"Agency Branding Updated","details":"Đổi nhận diện: NTH CRM","created":"2026-08-21T15:56:50.885Z","updated":"2026-08-21T15:56:50.885Z"}]</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63000011444092" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -1366,19 +1361,55 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[{"id":1,"name":"Thành phố Hà Nội","level":"City","parentId":null,"slug":"thanh-pho-ha-noi","code":"01","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":128,"name":"Tỉnh Cao Bằng","level":"City","parentId":null,"slug":"tinh-cao-bang","code":"04","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":185,"name":"Tỉnh Tuyên Quang","level":"City","parentId":null,"slug":"tinh-tuyen-quang","code":"08","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":310,"name":"Tỉnh Điện Biên","level":"City","parentId":null,"slug":"tinh-dien-bien","code":"11","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":356,"name":"Tỉnh Lai Châu","level":"City","parentId":null,"slug":"tinh-lai-chau","code":"12","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":395,"name":"Tỉnh Sơn La","level":"City","parentId":null,"slug":"tinh-son-la","code":"14","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":471,"name":"Tỉnh Lào Cai","level":"City","parentId":null,"slug":"tinh-lao-cai","code":"15","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":571,"name":"Tỉnh Thái Nguyên","level":"City","parentId":null,"slug":"tinh-thai-nguyen","code":"19","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":664,"name":"Tỉnh Lạng Sơn","level":"City","parentId":null,"slug":"tinh-lang-son","code":"20","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":730,"name":"Tỉnh Quảng Ninh","level":"City","parentId":null,"slug":"tinh-quang-ninh","code":"22","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":785,"name":"Tỉnh Bắc Ninh","level":"City","parentId":null,"slug":"tinh-bac-ninh","code":"24","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":885,"name":"Tỉnh Phú Thọ","level":"City","parentId":null,"slug":"tinh-phu-tho","code":"25","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1034,"name":"Thành phố Hải Phòng","level":"City","parentId":null,"slug":"thanh-pho-hai-phong","code":"31","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1149,"name":"Tỉnh Hưng Yên","level":"City","parentId":null,"slug":"tinh-hung-yen","code":"33","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1254,"name":"Tỉnh Ninh Bình","level":"City","parentId":null,"slug":"tinh-ninh-binh","code":"37","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1384,"name":"Tỉnh Thanh Hoá","level":"City","parentId":null,"slug":"tinh-thanh-hoa","code":"38","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1551,"name":"Tỉnh Nghệ An","level":"City","parentId":null,"slug":"tinh-nghe-an","code":"40","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1682,"name":"Tỉnh Hà Tĩnh","level":"City","parentId":null,"slug":"tinh-ha-tinh","code":"42","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1752,"name":"Tỉnh Quảng Trị","level":"City","parentId":null,"slug":"tinh-quang-tri","code":"44","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1831,"name":"Thành phố Huế","level":"City","parentId":null,"slug":"thanh-pho-hue","code":"46","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1872,"name":"Thành phố Đà Nẵng","level":"City","parentId":null,"slug":"thanh-pho-da-nang","code":"48","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":1967,"name":"Tỉnh Quảng Ngãi","level":"City","parentId":null,"slug":"tinh-quang-ngai","code":"51","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2064,"name":"Tỉnh Gia Lai","level":"City","parentId":null,"slug":"tinh-gia-lai","code":"52","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2200,"name":"Tỉnh Khánh Hoà","level":"City","parentId":null,"slug":"tinh-khanh-hoa","code":"56","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2266,"name":"Tỉnh Đắk Lắk","level":"City","parentId":null,"slug":"tinh-dak-lak","code":"66","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2369,"name":"Tỉnh Lâm Đồng","level":"City","parentId":null,"slug":"tinh-lam-dong","code":"68","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2494,"name":"Thành phố Đồng Nai","level":"City","parentId":null,"slug":"thanh-pho-dong-nai","code":"75","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2590,"name":"Thành phố Hồ Chí Minh","level":"City","parentId":null,"slug":"thanh-pho-ho-chi-minh","code":"79","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2759,"name":"Tỉnh Tây Ninh","level":"City","parentId":null,"slug":"tinh-tay-ninh","code":"80","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2856,"name":"Tỉnh Đồng Tháp","level":"City","parentId":null,"slug":"tinh-dong-thap","code":"82","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":2959,"name":"Tỉnh Vĩnh Long","level":"City","parentId":null,"slug":"tinh-vinh-long","code":"86","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":3084,"name":"Tỉnh An Giang","level":"City","parentId":null,"slug":"tinh-an-giang","code":"91","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":3187,"name":"Thành phố Cần Thơ","level":"City","parentId":null,"slug":"thanh-pho-can-tho","code":"92","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":3291,"name":"Tỉnh Cà Mau","level":"City","parentId":null,"slug":"tinh-ca-mau","code":"96","created":"2026-07-16T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"}]</t>
+          <t>[{"name":"Lahore","level":"City","parentId":null,"slug":"lahore","created":"2026-07-16T11:09:21.775Z","id":1,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Karachi","level":"City","parentId":null,"slug":"karachi","created":"2026-07-16T11:09:21.775Z","id":2,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Islamabad","level":"City","parentId":null,"slug":"islamabad","created":"2026-07-16T11:09:21.775Z","id":3,"updated":"2026-08-05T11:09:21.841Z"},{"name":"DHA Lahore","level":"Area","parentId":1,"slug":"dha-lahore","created":"2026-07-16T11:09:21.775Z","id":4,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Bahria Town","level":"Area","parentId":1,"slug":"bahria-town","created":"2026-07-16T11:09:21.775Z","id":5,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Gulberg","level":"Area","parentId":1,"slug":"gulberg","created":"2026-07-16T11:09:21.775Z","id":6,"updated":"2026-08-05T11:09:21.841Z"}]</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>[{"name":"DHA Karachi","level":"Area","parentId":2,"slug":"dha-karachi","created":"2026-07-17T11:09:21.775Z","id":7,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Clifton","level":"Area","parentId":2,"slug":"clifton","created":"2026-07-17T11:09:21.775Z","id":8,"updated":"2026-08-05T11:09:21.841Z"},{"name":"G-11","level":"Area","parentId":3,"slug":"g-11","created":"2026-07-17T11:09:21.775Z","id":9,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Bahria Enclave","level":"Area","parentId":3,"slug":"bahria-enclave","created":"2026-07-17T11:09:21.775Z","id":10,"updated":"2026-08-05T11:09:21.841Z"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>[{"id":2,"name":"Phường Ba Đình","level":"Area","parentId":1,"slug":"phuong-ba-dinh","code":"00004","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":3,"name":"Phường Ngọc Hà","level":"Area","parentId":1,"slug":"phuong-ngoc-ha","code":"00008","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":4,"name":"Phường Giảng Võ","level":"Area","parentId":1,"slug":"phuong-giang-vo","code":"00025","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":5,"name":"Phường Hoàn Kiếm","level":"Area","parentId":1,"slug":"phuong-hoan-kiem","code":"00070","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":6,"name":"Phường Cửa Nam","level":"Area","parentId":1,"slug":"phuong-cua-nam","code":"00082","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":7,"name":"Phường Phú Thượng","level":"Area","parentId":1,"slug":"phuong-phu-thuong","code":"00091","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":8,"name":"Phường Hồng Hà","level":"Area","parentId":1,"slug":"phuong-hong-ha","code":"00097","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":9,"name":"Phường Tây Hồ","level":"Area","parentId":1,"slug":"phuong-tay-ho","code":"00103","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":10,"name":"Phường Bồ Đề","level":"Area","parentId":1,"slug":"phuong-bo-de","code":"00118","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":11,"name":"Phường Việt Hưng","level":"Area","parentId":1,"slug":"phuong-viet-hung","code":"00127","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":12,"name":"Phường Phúc Lợi","level":"Area","parentId":1,"slug":"phuong-phuc-loi","code":"00136","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":13,"name":"Phường Long Biên","level":"Area","parentId":1,"slug":"phuong-long-bien","code":"00145","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":14,"name":"Phường Nghĩa Đô","level":"Area","parentId":1,"slug":"phuong-nghia-do","code":"00160","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":15,"name":"Phường Cầu Giấy","level":"Area","parentId":1,"slug":"phuong-cau-giay","code":"00166","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":16,"name":"Phường Yên Hoà","level":"Area","parentId":1,"slug":"phuong-yen-hoa","code":"00175","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":17,"name":"Phường Ô Chợ Dừa","level":"Area","parentId":1,"slug":"phuong-o-cho-dua","code":"00190","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":18,"name":"Phường Láng","level":"Area","parentId":1,"slug":"phuong-lang","code":"00199","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":19,"name":"Phường Văn Miếu - Quốc Tử Giám","level":"Area","parentId":1,"slug":"phuong-van-mieu-quoc-tu-giam","code":"00226","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":20,"name":"Phường Kim Liên","level":"Area","parentId":1,"slug":"phuong-kim-lien","code":"00229","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":21,"name":"Phường Đống Đa","level":"Area","parentId":1,"slug":"phuong-dong-da","code":"00235","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":22,"name":"Phường Hai Bà Trưng","level":"Area","parentId":1,"slug":"phuong-hai-ba-trung","code":"00256","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":23,"name":"Phường Vĩnh Tuy","level":"Area","parentId":1,"slug":"phuong-vinh-tuy","code":"00283","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":24,"name":"Phường Bạch Mai","level":"Area","parentId":1,"slug":"phuong-bach-mai","code":"00292","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":25,"name":"Phường Vĩnh Hưng","level":"Area","parentId":1,"slug":"phuong-vinh-hung","code":"00301","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":26,"name":"Phường Định Công","level":"Area","parentId":1,"slug":"phuong-dinh-cong","code":"00316","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":27,"name":"Phường Tương Mai","level":"Area","parentId":1,"slug":"phuong-tuong-mai","code":"00322","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":28,"name":"Phường Lĩnh Nam","level":"Area","parentId":1,"slug":"phuong-linh-nam","code":"00328","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":29,"name":"Phường Hoàng Mai","level":"Area","parentId":1,"slug":"phuong-hoang-mai","code":"00331","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":30,"name":"Phường Hoàng Liệt","level":"Area","parentId":1,"slug":"phuong-hoang-liet","code":"00337","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":31,"name":"Phường Yên Sở","level":"Area","parentId":1,"slug":"phuong-yen-so","code":"00340","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":32,"name":"Phường Phương Liệt","level":"Area","parentId":1,"slug":"phuong-phuong-liet","code":"00352","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":33,"name":"Phường Khương Đình","level":"Area","parentId":1,"slug":"phuong-khuong-dinh","code":"00364","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":34,"name":"Phường Thanh Xuân","level":"Area","parentId":1,"slug":"phuong-thanh-xuan","code":"00367","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":35,"name":"Xã Sóc Sơn","level":"Area","parentId":1,"slug":"xa-soc-son","code":"00376","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":36,"name":"Xã Kim Anh","level":"Area","parentId":1,"slug":"xa-kim-anh","code":"00382","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":37,"name":"Xã Trung Giã","level":"Area","parentId":1,"slug":"xa-trung-gia","code":"00385","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":38,"name":"Xã Đa Phúc","level":"Area","parentId":1,"slug":"xa-da-phuc","code":"00430","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":39,"name":"Xã Nội Bài","level":"Area","parentId":1,"slug":"xa-noi-bai","code":"00433","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":40,"name":"Xã Đông Anh","level":"Area","parentId":1,"slug":"xa-dong-anh","code":"00454","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":41,"name":"Xã Phúc Thịnh","level":"Area","parentId":1,"slug":"xa-phuc-thinh","code":"00466","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":42,"name":"Xã Thư Lâm","level":"Area","parentId":1,"slug":"xa-thu-lam","code":"00475","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":43,"name":"Xã Thiên Lộc","level":"Area","parentId":1,"slug":"xa-thien-loc","code":"00493","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":44,"name":"Xã Vĩnh Thanh","level":"Area","parentId":1,"slug":"xa-vinh-thanh","code":"00508","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":45,"name":"Xã Phù Đổng","level":"Area","parentId":1,"slug":"xa-phu-dong","code":"00541","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":46,"name":"Xã Thuận An","level":"Area","parentId":1,"slug":"xa-thuan-an","code":"00562","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":47,"name":"Xã Gia Lâm","level":"Area","parentId":1,"slug":"xa-gia-lam","code":"00565","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":48,"name":"Xã Bát Tràng","level":"Area","parentId":1,"slug":"xa-bat-trang","code":"00577","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":49,"name":"Phường Từ Liêm","level":"Area","parentId":1,"slug":"phuong-tu-liem","code":"00592","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":50,"name":"Phường Thượng Cát","level":"Area","parentId":1,"slug":"phuong-thuong-cat","code":"00598","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":51,"name":"Phường Đông Ngạc","level":"Area","parentId":1,"slug":"phuong-dong-ngac","code":"00602","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":52,"name":"Phường Xuân Đỉnh","level":"Area","parentId":1,"slug":"phuong-xuan-dinh","code":"00611","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":53,"name":"Phường Tây Tựu","level":"Area","parentId":1,"slug":"phuong-tay-tuu","code":"00613","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":54,"name":"Phường Phú Diễn","level":"Area","parentId":1,"slug":"phuong-phu-dien","code":"00619","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":55,"name":"Phường Xuân Phương","level":"Area","parentId":1,"slug":"phuong-xuan-phuong","code":"00622","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":56,"name":"Phường Tây Mỗ","level":"Area","parentId":1,"slug":"phuong-tay-mo","code":"00634","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":57,"name":"Phường Đại Mỗ","level":"Area","parentId":1,"slug":"phuong-dai-mo","code":"00637","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":58,"name":"Xã Thanh Trì","level":"Area","parentId":1,"slug":"xa-thanh-tri","code":"00640","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":59,"name":"Phường Thanh Liệt","level":"Area","parentId":1,"slug":"phuong-thanh-liet","code":"00643","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":60,"name":"Xã Đại Thanh","level":"Area","parentId":1,"slug":"xa-dai-thanh","code":"00664","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":61,"name":"Xã Ngọc Hồi","level":"Area","parentId":1,"slug":"xa-ngoc-hoi","code":"00679","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":62,"name":"Xã Nam Phù","level":"Area","parentId":1,"slug":"xa-nam-phu","code":"00685","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":63,"name":"Xã Yên Xuân","level":"Area","parentId":1,"slug":"xa-yen-xuan","code":"04930","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":64,"name":"Xã Quang Minh","level":"Area","parentId":1,"slug":"xa-quang-minh","code":"08974","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":65,"name":"Xã Yên Lãng","level":"Area","parentId":1,"slug":"xa-yen-lang","code":"08980","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":66,"name":"Xã Tiến Thắng","level":"Area","parentId":1,"slug":"xa-tien-thang","code":"08995","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":67,"name":"Xã Mê Linh","level":"Area","parentId":1,"slug":"xa-me-linh","code":"09022","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":68,"name":"Phường Kiến Hưng","level":"Area","parentId":1,"slug":"phuong-kien-hung","code":"09552","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":69,"name":"Phường Hà Đông","level":"Area","parentId":1,"slug":"phuong-ha-dong","code":"09556","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":70,"name":"Phường Yên Nghĩa","level":"Area","parentId":1,"slug":"phuong-yen-nghia","code":"09562","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":71,"name":"Phường Phú Lương","level":"Area","parentId":1,"slug":"phuong-phu-luong","code":"09568","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":72,"name":"Phường Sơn Tây","level":"Area","parentId":1,"slug":"phuong-son-tay","code":"09574","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":73,"name":"Phường Tùng Thiện","level":"Area","parentId":1,"slug":"phuong-tung-thien","code":"09604","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":74,"name":"Xã Đoài Phương","level":"Area","parentId":1,"slug":"xa-doai-phuong","code":"09616","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":75,"name":"Xã Quảng Oai","level":"Area","parentId":1,"slug":"xa-quang-oai","code":"09619","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":76,"name":"Xã Cổ Đô","level":"Area","parentId":1,"slug":"xa-co-do","code":"09634","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":77,"name":"Xã Minh Châu","level":"Area","parentId":1,"slug":"xa-minh-chau","code":"09661","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":78,"name":"Xã Vật Lại","level":"Area","parentId":1,"slug":"xa-vat-lai","code":"09664","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":79,"name":"Xã Bất Bạt","level":"Area","parentId":1,"slug":"xa-bat-bat","code":"09676","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":80,"name":"Xã Suối Hai","level":"Area","parentId":1,"slug":"xa-suoi-hai","code":"09694","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":81,"name":"Xã Ba Vì","level":"Area","parentId":1,"slug":"xa-ba-vi","code":"09700","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":82,"name":"Xã Yên Bài","level":"Area","parentId":1,"slug":"xa-yen-bai","code":"09706","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":83,"name":"Xã Phúc Thọ","level":"Area","parentId":1,"slug":"xa-phuc-tho","code":"09715","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":84,"name":"Xã Phúc Lộc","level":"Area","parentId":1,"slug":"xa-phuc-loc","code":"09739","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":85,"name":"Xã Hát Môn","level":"Area","parentId":1,"slug":"xa-hat-mon","code":"09772","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":86,"name":"Xã Đan Phượng","level":"Area","parentId":1,"slug":"xa-dan-phuong","code":"09784","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":87,"name":"Xã Liên Minh","level":"Area","parentId":1,"slug":"xa-lien-minh","code":"09787","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":88,"name":"Xã Ô Diên","level":"Area","parentId":1,"slug":"xa-o-dien","code":"09817","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":89,"name":"Xã Hoài Đức","level":"Area","parentId":1,"slug":"xa-hoai-duc","code":"09832","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":90,"name":"Xã Dương Hoà","level":"Area","parentId":1,"slug":"xa-duong-hoa","code":"09856","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":91,"name":"Xã Sơn Đồng","level":"Area","parentId":1,"slug":"xa-son-dong","code":"09871","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":92,"name":"Xã An Khánh","level":"Area","parentId":1,"slug":"xa-an-khanh","code":"09877","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":93,"name":"Phường Dương Nội","level":"Area","parentId":1,"slug":"phuong-duong-noi","code":"09886","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":94,"name":"Xã Quốc Oai","level":"Area","parentId":1,"slug":"xa-quoc-oai","code":"09895","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":95,"name":"Xã Kiều Phú","level":"Area","parentId":1,"slug":"xa-kieu-phu","code":"09910","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":96,"name":"Xã Hưng Đạo","level":"Area","parentId":1,"slug":"xa-hung-dao","code":"09931","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":97,"name":"Xã Phú Cát","level":"Area","parentId":1,"slug":"xa-phu-cat","code":"09952","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":98,"name":"Xã Thạch Thất","level":"Area","parentId":1,"slug":"xa-thach-that","code":"09955","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":99,"name":"Xã Hạ Bằng","level":"Area","parentId":1,"slug":"xa-ha-bang","code":"09982","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":100,"name":"Xã Hoà Lạc","level":"Area","parentId":1,"slug":"xa-hoa-lac","code":"09988","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":101,"name":"Xã Tây Phương","level":"Area","parentId":1,"slug":"xa-tay-phuong","code":"10003","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":102,"name":"Phường Chương Mỹ","level":"Area","parentId":1,"slug":"phuong-chuong-my","code":"10015","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":103,"name":"Xã Phú Nghĩa","level":"Area","parentId":1,"slug":"xa-phu-nghia","code":"10030","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":104,"name":"Xã Xuân Mai","level":"Area","parentId":1,"slug":"xa-xuan-mai","code":"10045","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":105,"name":"Xã Quảng Bị","level":"Area","parentId":1,"slug":"xa-quang-bi","code":"10072","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":106,"name":"Xã Trần Phú","level":"Area","parentId":1,"slug":"xa-tran-phu","code":"10081","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":107,"name":"Xã Hoà Phú","level":"Area","parentId":1,"slug":"xa-hoa-phu","code":"10096","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":108,"name":"Xã Thanh Oai","level":"Area","parentId":1,"slug":"xa-thanh-oai","code":"10114","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":109,"name":"Xã Bình Minh","level":"Area","parentId":1,"slug":"xa-binh-minh","code":"10126","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":110,"name":"Xã Tam Hưng","level":"Area","parentId":1,"slug":"xa-tam-hung","code":"10144","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":111,"name":"Xã Dân Hoà","level":"Area","parentId":1,"slug":"xa-dan-hoa","code":"10180","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":112,"name":"Xã Thường Tín","level":"Area","parentId":1,"slug":"xa-thuong-tin","code":"10183","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":113,"name":"Xã Hồng Vân","level":"Area","parentId":1,"slug":"xa-hong-van","code":"10210","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":114,"name":"Xã Thượng Phúc","level":"Area","parentId":1,"slug":"xa-thuong-phuc","code":"10231","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":115,"name":"Xã Chương Dương","level":"Area","parentId":1,"slug":"xa-chuong-duong","code":"10237","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":116,"name":"Xã Phú Xuyên","level":"Area","parentId":1,"slug":"xa-phu-xuyen","code":"10273","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":117,"name":"Xã Phượng Dực","level":"Area","parentId":1,"slug":"xa-phuong-duc","code":"10279","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":118,"name":"Xã Chuyên Mỹ","level":"Area","parentId":1,"slug":"xa-chuyen-my","code":"10330","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":119,"name":"Xã Đại Xuyên","level":"Area","parentId":1,"slug":"xa-dai-xuyen","code":"10342","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":120,"name":"Xã Vân Đình","level":"Area","parentId":1,"slug":"xa-van-dinh","code":"10354","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":121,"name":"Xã Ứng Thiên","level":"Area","parentId":1,"slug":"xa-ung-thien","code":"10369","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":122,"name":"Xã Ứng Hoà","level":"Area","parentId":1,"slug":"xa-ung-hoa","code":"10402","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":123,"name":"Xã Hoà Xá","level":"Area","parentId":1,"slug":"xa-hoa-xa","code":"10417","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":124,"name":"Xã Mỹ Đức","level":"Area","parentId":1,"slug":"xa-my-duc","code":"10441","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":125,"name":"Xã Phúc Sơn","level":"Area","parentId":1,"slug":"xa-phuc-son","code":"10459","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":126,"name":"Xã Hồng Sơn","level":"Area","parentId":1,"slug":"xa-hong-son","code":"10465","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":127,"name":"Xã Hương Sơn","level":"Area","parentId":1,"slug":"xa-huong-son","code":"10489","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":129,"name":"Phường Thục Phán","level":"Area","parentId":128,"slug":"phuong-thuc-phan","code":"01273","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":130,"name":"Phường Nùng Trí Cao","level":"Area","parentId":128,"slug":"phuong-nung-tri-cao","code":"01279","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":131,"name":"Phường Tân Giang","level":"Area","parentId":128,"slug":"phuong-tan-giang","code":"01288","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":132,"name":"Xã Bảo Lâm","level":"Area","parentId":128,"slug":"xa-bao-lam","code":"01290","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":133,"name":"Xã Lý Bôn","level":"Area","parentId":128,"slug":"xa-ly-bon","code":"01294","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":134,"name":"Xã Nam Quang","level":"Area","parentId":128,"slug":"xa-nam-quang","code":"01297","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":135,"name":"Xã Quảng Lâm","level":"Area","parentId":128,"slug":"xa-quang-lam","code":"01304","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":136,"name":"Xã Yên Thổ","level":"Area","parentId":128,"slug":"xa-yen-tho","code":"01318","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":137,"name":"Xã Bảo Lạc","level":"Area","parentId":128,"slug":"xa-bao-lac","code":"01321","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":138,"name":"Xã Cốc Pàng","level":"Area","parentId":128,"slug":"xa-coc-pang","code":"01324","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":139,"name":"Xã Cô Ba","level":"Area","parentId":128,"slug":"xa-co-ba","code":"01327","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":140,"name":"Xã Khánh Xuân","level":"Area","parentId":128,"slug":"xa-khanh-xuan","code":"01336","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":141,"name":"Xã Xuân Trường","level":"Area","parentId":128,"slug":"xa-xuan-truong","code":"01339","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":142,"name":"Xã Hưng Đạo","level":"Area","parentId":128,"slug":"xa-hung-dao","code":"01351","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":143,"name":"Xã Huy Giáp","level":"Area","parentId":128,"slug":"xa-huy-giap","code":"01354","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":144,"name":"Xã Sơn Lộ","level":"Area","parentId":128,"slug":"xa-son-lo","code":"01360","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":145,"name":"Xã Thông Nông","level":"Area","parentId":128,"slug":"xa-thong-nong","code":"01363","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":146,"name":"Xã Cần Yên","level":"Area","parentId":128,"slug":"xa-can-yen","code":"01366","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":147,"name":"Xã Thanh Long","level":"Area","parentId":128,"slug":"xa-thanh-long","code":"01387","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":148,"name":"Xã Trường Hà","level":"Area","parentId":128,"slug":"xa-truong-ha","code":"01392","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":149,"name":"Xã Lũng Nặm","level":"Area","parentId":128,"slug":"xa-lung-nam","code":"01393","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":150,"name":"Xã Tổng Cọt","level":"Area","parentId":128,"slug":"xa-tong-cot","code":"01414","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":151,"name":"Xã Hà Quảng","level":"Area","parentId":128,"slug":"xa-ha-quang","code":"01438","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":152,"name":"Xã Trà Lĩnh","level":"Area","parentId":128,"slug":"xa-tra-linh","code":"01447","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":153,"name":"Xã Quang Hán","level":"Area","parentId":128,"slug":"xa-quang-han","code":"01456","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":154,"name":"Xã Quang Trung","level":"Area","parentId":128,"slug":"xa-quang-trung","code":"01465","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":155,"name":"Xã Trùng Khánh","level":"Area","parentId":128,"slug":"xa-trung-khanh","code":"01477","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":156,"name":"Xã Đình Phong","level":"Area","parentId":128,"slug":"xa-dinh-phong","code":"01489","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":157,"name":"Xã Đàm Thuỷ","level":"Area","parentId":128,"slug":"xa-dam-thuy","code":"01501","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":158,"name":"Xã Đoài Dương","level":"Area","parentId":128,"slug":"xa-doai-duong","code":"01525","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":159,"name":"Xã Lý Quốc","level":"Area","parentId":128,"slug":"xa-ly-quoc","code":"01537","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":160,"name":"Xã Quang Long","level":"Area","parentId":128,"slug":"xa-quang-long","code":"01552","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":161,"name":"Xã Hạ Lang","level":"Area","parentId":128,"slug":"xa-ha-lang","code":"01558","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":162,"name":"Xã Vinh Quý","level":"Area","parentId":128,"slug":"xa-vinh-quy","code":"01561","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":163,"name":"Xã Quảng Uyên","level":"Area","parentId":128,"slug":"xa-quang-uyen","code":"01576","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":164,"name":"Xã Độc Lập","level":"Area","parentId":128,"slug":"xa-doc-lap","code":"01594","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":165,"name":"Xã Hạnh Phúc","level":"Area","parentId":128,"slug":"xa-hanh-phuc","code":"01618","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":166,"name":"Xã Bế Văn Đàn","level":"Area","parentId":128,"slug":"xa-be-van-dan","code":"01636","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":167,"name":"Xã Phục Hoà","level":"Area","parentId":128,"slug":"xa-phuc-hoa","code":"01648","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":168,"name":"Xã Hoà An","level":"Area","parentId":128,"slug":"xa-hoa-an","code":"01654","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":169,"name":"Xã Nam Tuấn","level":"Area","parentId":128,"slug":"xa-nam-tuan","code":"01660","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":170,"name":"Xã Nguyễn Huệ","level":"Area","parentId":128,"slug":"xa-nguyen-hue","code":"01699","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":171,"name":"Xã Bạch Đằng","level":"Area","parentId":128,"slug":"xa-bach-dang","code":"01708","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":172,"name":"Xã Nguyên Bình","level":"Area","parentId":128,"slug":"xa-nguyen-binh","code":"01726","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":173,"name":"Xã Tĩnh Túc","level":"Area","parentId":128,"slug":"xa-tinh-tuc","code":"01729","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":174,"name":"Xã Ca Thành","level":"Area","parentId":128,"slug":"xa-ca-thanh","code":"01738","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":175,"name":"Xã Minh Tâm","level":"Area","parentId":128,"slug":"xa-minh-tam","code":"01747","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":176,"name":"Xã Phan Thanh","level":"Area","parentId":128,"slug":"xa-phan-thanh","code":"01768","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":177,"name":"Xã Tam Kim","level":"Area","parentId":128,"slug":"xa-tam-kim","code":"01774","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":178,"name":"Xã Thành Công","level":"Area","parentId":128,"slug":"xa-thanh-cong","code":"01777","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":179,"name":"Xã Đông Khê","level":"Area","parentId":128,"slug":"xa-dong-khe","code":"01786","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":180,"name":"Xã Canh Tân","level":"Area","parentId":128,"slug":"xa-canh-tan","code":"01789","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":181,"name":"Xã Kim Đồng","level":"Area","parentId":128,"slug":"xa-kim-dong","code":"01792","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":182,"name":"Xã Minh Khai","level":"Area","parentId":128,"slug":"xa-minh-khai","code":"01795","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":183,"name":"Xã Thạch An","level":"Area","parentId":128,"slug":"xa-thach-an","code":"01807","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":184,"name":"Xã Đức Long","level":"Area","parentId":128,"slug":"xa-duc-long","code":"01822","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":186,"name":"Phường Hà Giang 2","level":"Area","parentId":185,"slug":"phuong-ha-giang-2","code":"00691","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":187,"name":"Phường Hà Giang 1","level":"Area","parentId":185,"slug":"phuong-ha-giang-1","code":"00694","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":188,"name":"Xã Ngọc Đường","level":"Area","parentId":185,"slug":"xa-ngoc-duong","code":"00700","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":189,"name":"Xã Phú Linh","level":"Area","parentId":185,"slug":"xa-phu-linh","code":"00706","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":190,"name":"Xã Lũng Cú","level":"Area","parentId":185,"slug":"xa-lung-cu","code":"00715","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":191,"name":"Xã Đồng Văn","level":"Area","parentId":185,"slug":"xa-dong-van","code":"00721","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":192,"name":"Xã Sà Phìn","level":"Area","parentId":185,"slug":"xa-sa-phin","code":"00733","created":"2026-07-18T11:09:21.775Z","updated":"2026-08-05T11:09:21.841Z"},{"id":193,"n</t>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[{"name":"Phase 5","level":"Society","parentId":4,"slug":"dha-lahore-phase-5","created":"2026-07-18T11:09:21.775Z","id":11,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Phase 6","level":"Society","parentId":4,"slug":"dha-lahore-phase-6","created":"2026-07-18T11:09:21.775Z","id":12,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Sector C","level":"Society","parentId":5,"slug":"bahria-town-sector-c","created":"2026-07-18T11:09:21.775Z","id":13,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Phase 8","level":"Society","parentId":7,"slug":"dha-karachi-phase-8","created":"2026-07-18T11:09:21.775Z","id":14,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Block 4","level":"Society","parentId":8,"slug":"clifton-block-4","created":"2026-07-18T11:09:21.775Z","id":15,"updated":"2026-08-05T11:09:21.841Z"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>[{"name":"Sector D","level":"Society","parentId":5,"slug":"bahria-town-sector-d","created":"2026-07-19T11:09:21.775Z","id":16,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Sector E","level":"Society","parentId":5,"slug":"bahria-town-sector-e","created":"2026-07-19T11:09:21.775Z","id":17,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Block 7","level":"Society","parentId":8,"slug":"clifton-block-7","created":"2026-07-19T11:09:21.775Z","id":18,"updated":"2026-08-05T11:09:21.841Z"}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>[{"name":"Phase 7","level":"Society","parentId":4,"slug":"dha-lahore-phase-7","created":"2026-07-20T11:09:21.775Z","id":19,"updated":"2026-08-05T11:09:21.841Z"},{"name":"Sector B","level":"Society","parentId":10,"slug":"bahria-enclave-sector-b","created":"2026-07-20T11:09:21.775Z","id":20,"updated":"2026-08-05T11:09:21.841Z"}]</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63000011444092" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -1466,7 +1497,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1019","title":"1 Bed Studio Gulberg","slug":"1-bed-studio-gulberg-19","description":"Furnished studio near the commercial strip — let through the CRM pipeline.","propertyType":"Flat","listingType":"Rent","status":"Rented","price":6110000,"rentFrequency":"Monthly","areaSize":51.1,"areaUnit":"Sq M","bedrooms":1,"bathrooms":1,"locationId":2591,"address":"Phường Thủ Dầu Một, Thành phố Hồ Chí Minh","latitude":null,"longitude":null,"ownerName":"Owner 19","ownerPhone":"03005000019","assignedAgent":"agent1","isFeatured":0,"viewsCount":88,"publishedAt":"2026-06-11T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re19a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re19b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re19c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,7,9],"createdBy":"agent1","created":"2026-06-10T11:09:23.919Z","id":19,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Thủ Dầu Một"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1019","title":"1 Bed Studio Gulberg","slug":"1-bed-studio-gulberg-19","description":"Furnished studio near the commercial strip — let through the CRM pipeline.","propertyType":"Flat","listingType":"Rent","status":"Rented","price":65000,"rentFrequency":"Monthly","areaSize":550,"areaUnit":"Sq Ft","bedrooms":1,"bathrooms":1,"locationId":6,"address":"Commercial strip","latitude":null,"longitude":null,"ownerName":"Owner 19","ownerPhone":"03005000019","assignedAgent":"agent1","isFeatured":0,"viewsCount":88,"publishedAt":"2026-06-11T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re19a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re19b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re19c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,7,9],"createdBy":"agent1","created":"2026-06-10T11:09:23.919Z","id":19,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1509,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1017","title":"126,46 m² Nhà phố liền kề","slug":"5-marla-house-phase-7-17","description":"Compact double-storey sold through the agency — retained for records and reporting.","propertyType":"House","listingType":"Sale","status":"Sold","price":2773000000,"rentFrequency":"","areaSize":126.46,"areaUnit":"Sq M","bedrooms":3,"bathrooms":3,"locationId":2,"address":"Phường Ba Đình, Thành phố Hà Nội","latitude":null,"longitude":null,"ownerName":"Owner 17","ownerPhone":"03005000017","assignedAgent":"agent2","isFeatured":0,"viewsCount":210,"publishedAt":"2026-07-12T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re17a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re17b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re17c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2],"createdBy":"agent3","created":"2026-07-11T11:09:23.919Z","id":17,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hà Nội › Phường Ba Đình"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1017","title":"5 Marla House Phase 7","slug":"5-marla-house-phase-7-17","description":"Compact double-storey sold through the agency — retained for records and reporting.","propertyType":"House","listingType":"Sale","status":"Sold","price":29500000,"rentFrequency":"","areaSize":5,"areaUnit":"Marla","bedrooms":3,"bathrooms":3,"locationId":19,"address":"Phase 7","latitude":null,"longitude":null,"ownerName":"Owner 17","ownerPhone":"03005000017","assignedAgent":"agent3","isFeatured":0,"viewsCount":210,"publishedAt":"2026-07-12T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re17a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re17b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re17c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2],"createdBy":"agent3","created":"2026-07-11T11:09:23.919Z","id":17,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1521,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-KAR-1011","title":"505,86 m² House DHA Karachi","slug":"1-kanal-house-dha-karachi-11","description":"Architect-designed family home, sold through the agency — kept for record and reporting.","propertyType":"House","listingType":"Sale","status":"Sold","price":10340000000,"rentFrequency":"","areaSize":505.86,"areaUnit":"Sq M","bedrooms":6,"bathrooms":6,"locationId":2592,"address":"Phường Phú Lợi, Thành phố Hồ Chí Minh","latitude":24.791,"longitude":67.1189,"ownerName":"Owner 11","ownerPhone":"03005000011","assignedAgent":"agent2","isFeatured":0,"viewsCount":385,"publishedAt":"2026-07-21T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re11a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re11b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re11c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,6],"createdBy":"admin","created":"2026-07-20T11:09:23.919Z","id":11,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Phú Lợi"}]</t>
+          <t>[{"referenceCode":"RS-KAR-1011","title":"1 Kanal House DHA Karachi","slug":"1-kanal-house-dha-karachi-11","description":"Architect-designed family home, sold through the agency — kept for record and reporting.","propertyType":"House","listingType":"Sale","status":"Sold","price":110000000,"rentFrequency":"","areaSize":1,"areaUnit":"Kanal","bedrooms":6,"bathrooms":6,"locationId":14,"address":"Phase 8","latitude":24.791,"longitude":67.1189,"ownerName":"Owner 11","ownerPhone":"03005000011","assignedAgent":"agent2","isFeatured":0,"viewsCount":385,"publishedAt":"2026-07-21T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re11a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re11b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re11c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,6],"createdBy":"admin","created":"2026-07-20T11:09:23.919Z","id":11,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1533,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1001","title":"252,93 m² Modern Nhà phố liền kề","slug":"10-marla-modern-house-phase-5-1","description":"Brand new double-storey house with imported fittings, solid wood doors and a landscaped lawn. Walking distance to the main park and commercial area.","propertyType":"House","listingType":"Sale","status":"Available","price":4230000000,"rentFrequency":"","areaSize":252.93,"areaUnit":"Sq M","bedrooms":4,"bathrooms":5,"locationId":1873,"address":"Phường Hải Vân, Thành phố Đà Nẵng","latitude":31.4676,"longitude":74.4107,"ownerName":"Owner 1","ownerPhone":"03005000001","assignedAgent":"agent1","isFeatured":1,"viewsCount":246,"publishedAt":"2026-07-24T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re1a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re1b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re1c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,4,6,10],"createdBy":"admin","created":"2026-07-22T11:09:23.919Z","id":1,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Đà Nẵng › Phường Hải Vân"},{"referenceCode":"RS-LAH-1010","title":"Upper Portion 252,93 m² Phase 5","slug":"upper-portion-10-marla-phase-5-10","description":"Separate-entrance upper portion with 3 beds and servant room. Rented out via the CRM pipeline.","propertyType":"Upper Portion","listingType":"Rent","status":"Rented","price":8930000,"rentFrequency":"Monthly","areaSize":252.93,"areaUnit":"Sq M","bedrooms":3,"bathrooms":3,"locationId":3,"address":"Phường Ngọc Hà, Thành phố Hà Nội","latitude":31.4659,"longitude":74.409,"ownerName":"Owner 10","ownerPhone":"03005000010","assignedAgent":"agent1","isFeatured":0,"viewsCount":203,"publishedAt":"2026-07-23T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re10a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re10b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re10c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10],"createdBy":"manager1","created":"2026-07-22T11:09:23.919Z","id":10,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hà Nội › Phường Ngọc Hà"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1001","title":"10 Marla Modern House Phase 5","slug":"10-marla-modern-house-phase-5-1","description":"Brand new double-storey house with imported fittings, solid wood doors and a landscaped lawn. Walking distance to the main park and commercial area.","propertyType":"House","listingType":"Sale","status":"Available","price":45000000,"rentFrequency":"","areaSize":10,"areaUnit":"Marla","bedrooms":4,"bathrooms":5,"locationId":11,"address":"Street 12, Phase 5","latitude":31.4676,"longitude":74.4107,"ownerName":"Owner 1","ownerPhone":"03005000001","assignedAgent":"agent1","isFeatured":1,"viewsCount":245,"publishedAt":"2026-07-24T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re1a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re1b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re1c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,4,6,10],"createdBy":"admin","created":"2026-07-22T11:09:23.919Z","id":1,"updated":"2026-08-05T11:09:23.965Z"},{"referenceCode":"RS-LAH-1010","title":"Upper Portion 10 Marla Phase 5","slug":"upper-portion-10-marla-phase-5-10","description":"Separate-entrance upper portion with 3 beds and servant room. Rented out via the CRM pipeline.","propertyType":"Upper Portion","listingType":"Rent","status":"Rented","price":95000,"rentFrequency":"Monthly","areaSize":10,"areaUnit":"Marla","bedrooms":3,"bathrooms":3,"locationId":11,"address":"Street 9, Phase 5","latitude":31.4659,"longitude":74.409,"ownerName":"Owner 10","ownerPhone":"03005000010","assignedAgent":"agent1","isFeatured":0,"viewsCount":203,"publishedAt":"2026-07-23T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re10a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re10b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re10c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10],"createdBy":"manager1","created":"2026-07-22T11:09:23.919Z","id":10,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1545,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1002","title":"126,46 m² Brand New Nhà phố liền kề","slug":"5-marla-brand-new-house-phase-6-2","description":"Stylish 126,46 m² house on a 40ft road — ideal first home with modern kitchen and 3 spacious bedrooms.","propertyType":"House","listingType":"Sale","status":"Available","price":2585000000,"rentFrequency":"","areaSize":126.46,"areaUnit":"Sq M","bedrooms":3,"bathrooms":4,"locationId":2593,"address":"Phường Bình Dương, Thành phố Hồ Chí Minh","latitude":31.4832,"longitude":74.4421,"ownerName":"Owner 2","ownerPhone":"03005000002","assignedAgent":"agent2","isFeatured":1,"viewsCount":189,"publishedAt":"2026-07-25T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re2a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re2b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re2c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10],"createdBy":"manager1","created":"2026-07-23T11:09:23.919Z","id":2,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Bình Dương"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1002","title":"5 Marla Brand New House Phase 6","slug":"5-marla-brand-new-house-phase-6-2","description":"Stylish 5 marla house on a 40ft road — ideal first home with modern kitchen and 3 spacious bedrooms.","propertyType":"House","listingType":"Sale","status":"Available","price":27500000,"rentFrequency":"","areaSize":5,"areaUnit":"Marla","bedrooms":3,"bathrooms":4,"locationId":12,"address":"Block C, Phase 6","latitude":31.4832,"longitude":74.4421,"ownerName":"Owner 2","ownerPhone":"03005000002","assignedAgent":"agent2","isFeatured":1,"viewsCount":189,"publishedAt":"2026-07-25T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re2a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re2b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re2c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10],"createdBy":"manager1","created":"2026-07-23T11:09:23.919Z","id":2,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1557,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1003","title":"505,86 m² Luxury Villa Sector C","slug":"1-kanal-luxury-villa-sector-c-3","description":"Designer villa with swimming pool, home theatre, basement and servant quarters. Facing park, fully furnished.","propertyType":"House","listingType":"Sale","status":"Reserved","price":7755000000,"rentFrequency":"","areaSize":505.86,"areaUnit":"Sq M","bedrooms":5,"bathrooms":6,"locationId":1035,"address":"Phường Thành Đông, Thành phố Hải Phòng","latitude":31.3684,"longitude":74.1801,"ownerName":"Owner 3","ownerPhone":"03005000003","assignedAgent":"agent1","isFeatured":0,"viewsCount":312,"publishedAt":"2026-07-26T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re3a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re3b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re3c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,5,6,9,11],"createdBy":"admin","created":"2026-07-24T11:09:23.919Z","id":3,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hải Phòng › Phường Thành Đông"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1003","title":"1 Kanal Luxury Villa Sector C","slug":"1-kanal-luxury-villa-sector-c-3","description":"Designer villa with swimming pool, home theatre, basement and servant quarters. Facing park, fully furnished.","propertyType":"House","listingType":"Sale","status":"Reserved","price":82500000,"rentFrequency":"","areaSize":1,"areaUnit":"Kanal","bedrooms":5,"bathrooms":6,"locationId":13,"address":"Sector C, Main Boulevard","latitude":31.3684,"longitude":74.1801,"ownerName":"Owner 3","ownerPhone":"03005000003","assignedAgent":"agent1","isFeatured":0,"viewsCount":312,"publishedAt":"2026-07-26T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re3a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re3b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re3c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,5,6,9,11],"createdBy":"admin","created":"2026-07-24T11:09:23.919Z","id":3,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1569,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1004","title":"2 Bed Apartment Gulberg","slug":"2-bed-apartment-gulberg-4","description":"Well-maintained apartment near Main Market with lift, standby generator and 24/7 security.","propertyType":"Flat","listingType":"Rent","status":"Available","price":11750000,"rentFrequency":"Monthly","areaSize":111.48,"areaUnit":"Sq M","bedrooms":2,"bathrooms":2,"locationId":4,"address":"Phường Giảng Võ, Thành phố Hà Nội","latitude":31.5102,"longitude":74.3441,"ownerName":"Owner 4","ownerPhone":"03005000004","assignedAgent":"agent2","isFeatured":0,"viewsCount":98,"publishedAt":"2026-07-27T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re4a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re4b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re4c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,6,7],"createdBy":"manager1","created":"2026-07-26T11:09:23.919Z","id":4,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hà Nội › Phường Giảng Võ"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1004","title":"2 Bed Apartment Gulberg","slug":"2-bed-apartment-gulberg-4","description":"Well-maintained apartment near Main Market with lift, standby generator and 24/7 security.","propertyType":"Flat","listingType":"Rent","status":"Available","price":125000,"rentFrequency":"Monthly","areaSize":1200,"areaUnit":"Sq Ft","bedrooms":2,"bathrooms":2,"locationId":6,"address":"Main Market vicinity","latitude":31.5102,"longitude":74.3441,"ownerName":"Owner 4","ownerPhone":"03005000004","assignedAgent":"agent3","isFeatured":0,"viewsCount":98,"publishedAt":"2026-07-27T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re4a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re4b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re4c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,6,7],"createdBy":"manager1","created":"2026-07-26T11:09:23.919Z","id":4,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1581,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-KAR-1005","title":"418,06 m² Biệt thự sân vườn","slug":"500-sq-yd-bungalow-phase-8-5","description":"Owner-built bungalow with basement, roof-top terrace and separate servant block. Prime Phase 8 location.","propertyType":"House","listingType":"Sale","status":"Available","price":8930000000,"rentFrequency":"","areaSize":418.06,"areaUnit":"Sq M","bedrooms":5,"bathrooms":5,"locationId":2594,"address":"Phường Phú An, Thành phố Hồ Chí Minh","latitude":24.7896,"longitude":67.1215,"ownerName":"Owner 5","ownerPhone":"03005000005","assignedAgent":"agent2","isFeatured":1,"viewsCount":426,"publishedAt":"2026-07-28T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re5a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re5b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re5c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,6,11],"createdBy":"admin","created":"2026-07-27T11:09:23.919Z","id":5,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Phú An"}]</t>
+          <t>[{"referenceCode":"RS-KAR-1005","title":"500 Sq Yd Bungalow Phase 8","slug":"500-sq-yd-bungalow-phase-8-5","description":"Owner-built bungalow with basement, roof-top terrace and separate servant block. Prime Phase 8 location.","propertyType":"House","listingType":"Sale","status":"Available","price":95000000,"rentFrequency":"","areaSize":500,"areaUnit":"Sq Yd","bedrooms":5,"bathrooms":5,"locationId":14,"address":"Phase 8, near park","latitude":24.7896,"longitude":67.1215,"ownerName":"Owner 5","ownerPhone":"03005000005","assignedAgent":"agent2","isFeatured":1,"viewsCount":421,"publishedAt":"2026-07-28T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re5a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re5b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re5c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,6,11],"createdBy":"admin","created":"2026-07-27T11:09:23.919Z","id":5,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1593,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-KAR-1006","title":"3 Bed Sea View Apartment Block 4","slug":"3-bed-sea-view-apartment-block-4-6","description":"High-floor apartment with open sea view, gym and community pool. Fully furnished, ready to move.","propertyType":"Flat","listingType":"Rent","status":"Available","price":17390000,"rentFrequency":"Monthly","areaSize":195.1,"areaUnit":"Sq M","bedrooms":3,"bathrooms":3,"locationId":1874,"address":"Phường Liên Chiểu, Thành phố Đà Nẵng","latitude":24.8138,"longitude":67.03,"ownerName":"Owner 6","ownerPhone":"03005000006","assignedAgent":"agent2","isFeatured":0,"viewsCount":156,"publishedAt":"2026-07-29T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re6a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re6b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re6c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,5,6,7,9,12],"createdBy":"manager1","created":"2026-07-28T11:09:23.919Z","id":6,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Đà Nẵng › Phường Liên Chiểu"},{"referenceCode":"RS-ISL-1007","title":"252,93 m² Double Storey G-11","slug":"10-marla-double-storey-g-11-7","description":"Solid construction near Markaz — was live, owner paused the sale (withdrawn from portal).","propertyType":"House","listingType":"Sale","status":"Withdrawn","price":4935000000,"rentFrequency":"","areaSize":252.93,"areaUnit":"Sq M","bedrooms":5,"bathrooms":4,"locationId":5,"address":"Phường Hoàn Kiếm, Thành phố Hà Nội","latitude":33.6693,"longitude":72.9971,"ownerName":"Owner 7","ownerPhone":"03005000007","assignedAgent":"agent1","isFeatured":0,"viewsCount":134,"publishedAt":"2026-07-29T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re7a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re7b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re7c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10],"createdBy":"admin","created":"2026-07-28T11:09:23.919Z","id":7,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hà Nội › Phường Hoàn Kiếm"}]</t>
+          <t>[{"referenceCode":"RS-KAR-1006","title":"3 Bed Sea View Apartment Block 4","slug":"3-bed-sea-view-apartment-block-4-6","description":"High-floor apartment with open sea view, gym and community pool. Fully furnished, ready to move.","propertyType":"Flat","listingType":"Rent","status":"Available","price":185000,"rentFrequency":"Monthly","areaSize":2100,"areaUnit":"Sq Ft","bedrooms":3,"bathrooms":3,"locationId":15,"address":"Block 4, seafront tower","latitude":24.8138,"longitude":67.03,"ownerName":"Owner 6","ownerPhone":"03005000006","assignedAgent":"agent3","isFeatured":0,"viewsCount":156,"publishedAt":"2026-07-29T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re6a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re6b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re6c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,5,6,7,9,12],"createdBy":"manager1","created":"2026-07-28T11:09:23.919Z","id":6,"updated":"2026-08-05T11:09:23.965Z"},{"referenceCode":"RS-ISL-1007","title":"10 Marla Double Storey G-11","slug":"10-marla-double-storey-g-11-7","description":"Solid construction near Markaz — was live, owner paused the sale (withdrawn from portal).","propertyType":"House","listingType":"Sale","status":"Withdrawn","price":52500000,"rentFrequency":"","areaSize":10,"areaUnit":"Marla","bedrooms":5,"bathrooms":4,"locationId":9,"address":"G-11/3","latitude":33.6693,"longitude":72.9971,"ownerName":"Owner 7","ownerPhone":"03005000007","assignedAgent":"agent1","isFeatured":0,"viewsCount":134,"publishedAt":"2026-07-29T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re7a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re7b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re7c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10],"createdBy":"admin","created":"2026-07-28T11:09:23.919Z","id":7,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1605,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-ISL-1008","title":"126,46 m² Plot Bahria Enclave","slug":"5-marla-plot-bahria-enclave-8","description":"Level, possession-ready plot on a 30ft road — all dues clear, ideal for immediate construction.","propertyType":"Plot","listingType":"Sale","status":"Reserved","price":921200000,"rentFrequency":"","areaSize":126.46,"areaUnit":"Sq M","bedrooms":null,"bathrooms":null,"locationId":2595,"address":"Phường Chánh Hiệp, Thành phố Hồ Chí Minh","latitude":33.6844,"longitude":73.1338,"ownerName":"Owner 8","ownerPhone":"03005000008","assignedAgent":"agent2","isFeatured":0,"viewsCount":89,"publishedAt":"2026-07-30T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re8a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re8b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re8c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[8],"createdBy":"manager1","created":"2026-07-29T11:09:23.919Z","id":8,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Chánh Hiệp"}]</t>
+          <t>[{"referenceCode":"RS-ISL-1008","title":"5 Marla Plot Bahria Enclave","slug":"5-marla-plot-bahria-enclave-8","description":"Level, possession-ready plot on a 30ft road — all dues clear, ideal for immediate construction.","propertyType":"Plot","listingType":"Sale","status":"Reserved","price":9800000,"rentFrequency":"","areaSize":5,"areaUnit":"Marla","bedrooms":null,"bathrooms":null,"locationId":10,"address":"Sector A","latitude":33.6844,"longitude":73.1338,"ownerName":"Owner 8","ownerPhone":"03005000008","assignedAgent":"agent2","isFeatured":0,"viewsCount":87,"publishedAt":"2026-07-30T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re8a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re8b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re8c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[8],"createdBy":"manager1","created":"2026-07-29T11:09:23.919Z","id":8,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1617,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1009","title":"Commercial Shop Gulberg Main Boulevard","slug":"commercial-shop-gulberg-main-boulevard-9","description":"Ground-floor shop with wide frontage on the main boulevard — high footfall, ideal for retail brands.","propertyType":"Shop","listingType":"Rent","status":"Rented","price":32900000,"rentFrequency":"Monthly","areaSize":74.32,"areaUnit":"Sq M","bedrooms":null,"bathrooms":1,"locationId":6,"address":"Phường Cửa Nam, Thành phố Hà Nội","latitude":31.5152,"longitude":74.3481,"ownerName":"Owner 9","ownerPhone":"03005000009","assignedAgent":"agent2","isFeatured":0,"viewsCount":76,"publishedAt":"2026-07-31T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re9a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re9b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re9c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,6],"createdBy":"admin","created":"2026-07-30T11:09:23.919Z","id":9,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hà Nội › Phường Cửa Nam"},{"referenceCode":"RS-LAH-1013","title":"177,05 m² Nhà phố liền kề","slug":"7-marla-house-phase-6-13","description":"Well-built family home on a quiet street — solar-ready wiring and a small lawn at the back.","propertyType":"House","listingType":"Sale","status":"Available","price":3149000000,"rentFrequency":"","areaSize":177.05,"areaUnit":"Sq M","bedrooms":4,"bathrooms":4,"locationId":2591,"address":"Phường Thủ Dầu Một, Thành phố Hồ Chí Minh","latitude":null,"longitude":null,"ownerName":"Owner 13","ownerPhone":"03005000013","assignedAgent":"agent1","isFeatured":0,"viewsCount":64,"publishedAt":"2026-07-31T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re13a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re13b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re13c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10,14],"createdBy":"agent1","created":"2026-07-30T11:09:23.919Z","id":13,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Thủ Dầu Một"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1009","title":"Commercial Shop Gulberg Main Boulevard","slug":"commercial-shop-gulberg-main-boulevard-9","description":"Ground-floor shop with wide frontage on the main boulevard — high footfall, ideal for retail brands.","propertyType":"Shop","listingType":"Rent","status":"Rented","price":350000,"rentFrequency":"Monthly","areaSize":800,"areaUnit":"Sq Ft","bedrooms":null,"bathrooms":1,"locationId":6,"address":"Main Boulevard","latitude":31.5152,"longitude":74.3481,"ownerName":"Owner 9","ownerPhone":"03005000009","assignedAgent":"agent3","isFeatured":0,"viewsCount":76,"publishedAt":"2026-07-31T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re9a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re9b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re9c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,6],"createdBy":"admin","created":"2026-07-30T11:09:23.919Z","id":9,"updated":"2026-08-05T11:09:23.965Z"},{"referenceCode":"RS-LAH-1013","title":"7 Marla House Phase 6","slug":"7-marla-house-phase-6-13","description":"Well-built family home on a quiet street — solar-ready wiring and a small lawn at the back.","propertyType":"House","listingType":"Sale","status":"Available","price":33500000,"rentFrequency":"","areaSize":7,"areaUnit":"Marla","bedrooms":4,"bathrooms":4,"locationId":12,"address":"Street 5, Phase 6","latitude":null,"longitude":null,"ownerName":"Owner 13","ownerPhone":"03005000013","assignedAgent":"agent1","isFeatured":0,"viewsCount":64,"publishedAt":"2026-07-31T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re13a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re13b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re13c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,10,14],"createdBy":"agent1","created":"2026-07-30T11:09:23.919Z","id":13,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1629,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-KAR-1014","title":"2 Bed Apartment Block 7","slug":"2-bed-apartment-block-7-14","description":"Mid-floor apartment with lift access and standby power — walking distance to the park.","propertyType":"Flat","listingType":"Rent","status":"Available","price":8930000,"rentFrequency":"Monthly","areaSize":102.19,"areaUnit":"Sq M","bedrooms":2,"bathrooms":2,"locationId":2,"address":"Phường Ba Đình, Thành phố Hà Nội","latitude":null,"longitude":null,"ownerName":"Owner 14","ownerPhone":"03005000014","assignedAgent":"agent2","isFeatured":0,"viewsCount":41,"publishedAt":"2026-07-31T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re14a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re14b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re14c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,6,7],"createdBy":"agent2","created":"2026-07-31T11:09:23.919Z","id":14,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hà Nội › Phường Ba Đình"}]</t>
+          <t>[{"referenceCode":"RS-KAR-1014","title":"2 Bed Apartment Block 7","slug":"2-bed-apartment-block-7-14","description":"Mid-floor apartment with lift access and standby power — walking distance to the park.","propertyType":"Flat","listingType":"Rent","status":"Available","price":95000,"rentFrequency":"Monthly","areaSize":1100,"areaUnit":"Sq Ft","bedrooms":2,"bathrooms":2,"locationId":18,"address":"Block 7","latitude":null,"longitude":null,"ownerName":"Owner 14","ownerPhone":"03005000014","assignedAgent":"agent2","isFeatured":0,"viewsCount":41,"publishedAt":"2026-07-31T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re14a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re14b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re14c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,6,7],"createdBy":"agent2","created":"2026-07-31T11:09:23.919Z","id":14,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1641,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-ISL-1015","title":"202,34 m² Plot Sector B","slug":"8-marla-plot-sector-b-15","description":"Level plot near the main gate — all development charges paid, ready for possession.","propertyType":"Plot","listingType":"Sale","status":"Available","price":1175000000,"rentFrequency":"","areaSize":202.34,"areaUnit":"Sq M","bedrooms":null,"bathrooms":null,"locationId":2592,"address":"Phường Phú Lợi, Thành phố Hồ Chí Minh","latitude":null,"longitude":null,"ownerName":"Owner 15","ownerPhone":"03005000015","assignedAgent":"agent2","isFeatured":0,"viewsCount":34,"publishedAt":"2026-08-01T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re15a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re15b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re15c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[8],"createdBy":"agent3","created":"2026-08-01T11:09:23.919Z","id":15,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Phú Lợi"},{"referenceCode":"RS-LAH-1016","title":"Office Floor Gulberg Boulevard","slug":"office-floor-gulberg-boulevard-16","description":"Open-plan office floor with dedicated parking and backup power — ideal for a software house.","propertyType":"Office","listingType":"Rent","status":"Available","price":25850000,"rentFrequency":"Monthly","areaSize":222.97,"areaUnit":"Sq M","bedrooms":null,"bathrooms":2,"locationId":1873,"address":"Phường Hải Vân, Thành phố Đà Nẵng","latitude":null,"longitude":null,"ownerName":"Owner 16","ownerPhone":"03005000016","assignedAgent":"agent2","isFeatured":0,"viewsCount":58,"publishedAt":"2026-08-01T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re16a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re16b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re16c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,6,7,15],"createdBy":"manager1","created":"2026-08-01T11:09:23.919Z","id":16,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Đà Nẵng › Phường Hải Vân"}]</t>
+          <t>[{"referenceCode":"RS-ISL-1015","title":"8 Marla Plot Sector B","slug":"8-marla-plot-sector-b-15","description":"Level plot near the main gate — all development charges paid, ready for possession.","propertyType":"Plot","listingType":"Sale","status":"Available","price":12500000,"rentFrequency":"","areaSize":8,"areaUnit":"Marla","bedrooms":null,"bathrooms":null,"locationId":20,"address":"Sector B","latitude":null,"longitude":null,"ownerName":"Owner 15","ownerPhone":"03005000015","assignedAgent":"agent3","isFeatured":0,"viewsCount":33,"publishedAt":"2026-08-01T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re15a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re15b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re15c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[8],"createdBy":"agent3","created":"2026-08-01T11:09:23.919Z","id":15,"updated":"2026-08-05T11:09:23.965Z"},{"referenceCode":"RS-LAH-1016","title":"Office Floor Gulberg Boulevard","slug":"office-floor-gulberg-boulevard-16","description":"Open-plan office floor with dedicated parking and backup power — ideal for a software house.","propertyType":"Office","listingType":"Rent","status":"Available","price":275000,"rentFrequency":"Monthly","areaSize":2400,"areaUnit":"Sq Ft","bedrooms":null,"bathrooms":2,"locationId":6,"address":"Main Boulevard","latitude":null,"longitude":null,"ownerName":"Owner 16","ownerPhone":"03005000016","assignedAgent":"agent2","isFeatured":0,"viewsCount":58,"publishedAt":"2026-08-01T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re16a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re16b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re16c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,6,7,15],"createdBy":"manager1","created":"2026-08-01T11:09:23.919Z","id":16,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1653,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-KAR-1018","title":"250,84 m² Nhà phố liền kề","slug":"300-sq-yd-house-phase-8-18","description":"Corner house with a sea-breeze terrace — recently renovated kitchen and bathrooms.","propertyType":"House","listingType":"Sale","status":"Available","price":6110000000,"rentFrequency":"","areaSize":250.84,"areaUnit":"Sq M","bedrooms":4,"bathrooms":5,"locationId":3,"address":"Phường Ngọc Hà, Thành phố Hà Nội","latitude":null,"longitude":null,"ownerName":"Owner 18","ownerPhone":"03005000018","assignedAgent":"agent2","isFeatured":1,"viewsCount":153,"publishedAt":"2026-08-02T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re18a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re18b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re18c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,4,6,18],"createdBy":"agent2","created":"2026-08-02T11:09:23.919Z","id":18,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hà Nội › Phường Ngọc Hà"}]</t>
+          <t>[{"referenceCode":"RS-KAR-1018","title":"300 Sq Yd House Phase 8","slug":"300-sq-yd-house-phase-8-18","description":"Corner house with a sea-breeze terrace — recently renovated kitchen and bathrooms.","propertyType":"House","listingType":"Sale","status":"Available","price":65000000,"rentFrequency":"","areaSize":300,"areaUnit":"Sq Yd","bedrooms":4,"bathrooms":5,"locationId":14,"address":"Phase 8","latitude":null,"longitude":null,"ownerName":"Owner 18","ownerPhone":"03005000018","assignedAgent":"agent2","isFeatured":1,"viewsCount":149,"publishedAt":"2026-08-02T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re18a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re18b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re18c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,4,6,18],"createdBy":"agent2","created":"2026-08-02T11:09:23.919Z","id":18,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1665,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-ISL-1020","title":"Farm House Sector B","slug":"farm-house-sector-b-20","description":"2.023,43 m² farm house with lawns, pool and staff quarters — event-ready with ample parking.","propertyType":"Farm House","listingType":"Sale","status":"Available","price":13630000000,"rentFrequency":"","areaSize":2023.43,"areaUnit":"Sq M","bedrooms":6,"bathrooms":7,"locationId":2593,"address":"Phường Bình Dương, Thành phố Hồ Chí Minh","latitude":null,"longitude":null,"ownerName":"Owner 20","ownerPhone":"03005000020","assignedAgent":"agent2","isFeatured":0,"viewsCount":176,"publishedAt":"2026-08-03T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re20a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re20b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re20c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,5,6],"createdBy":"admin","created":"2026-08-03T11:09:23.919Z","id":20,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hồ Chí Minh › Phường Bình Dương"}]</t>
+          <t>[{"referenceCode":"RS-ISL-1020","title":"Farm House Sector B","slug":"farm-house-sector-b-20","description":"4 kanal farm house with lawns, pool and staff quarters — event-ready with ample parking.","propertyType":"Farm House","listingType":"Sale","status":"Available","price":145000000,"rentFrequency":"","areaSize":4,"areaUnit":"Kanal","bedrooms":6,"bathrooms":7,"locationId":20,"address":"Sector B","latitude":null,"longitude":null,"ownerName":"Owner 20","ownerPhone":"03005000020","assignedAgent":"agent3","isFeatured":0,"viewsCount":176,"publishedAt":"2026-08-03T11:09:23.919Z","images":[{"url":"https://picsum.photos/seed/re20a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re20b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re20c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2,3,4,5,6],"createdBy":"admin","created":"2026-08-03T11:09:23.919Z","id":20,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1646,19 +1677,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[{"referenceCode":"RS-LAH-1012","title":"202,34 m² House Bahria Sector C","slug":"8-marla-house-bahria-sector-c-12","description":"Listing being prepared — photos and owner documents pending. Not yet on the public portal.","propertyType":"House","listingType":"Sale","status":"Draft","price":2914000000,"rentFrequency":"","areaSize":202.34,"areaUnit":"Sq M","bedrooms":4,"bathrooms":4,"locationId":1035,"address":"Phường Thành Đông, Thành phố Hải Phòng","latitude":31.3702,"longitude":74.1855,"ownerName":"Owner 12","ownerPhone":"03005000012","assignedAgent":"agent2","isFeatured":0,"viewsCount":0,"publishedAt":null,"images":[{"url":"https://picsum.photos/seed/re12a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re12b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re12c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2],"createdBy":"agent3","created":"2026-08-04T11:09:23.919Z","id":12,"updated":"2026-08-05T11:09:23.965Z","locationPath":"Thành phố Hải Phòng › Phường Thành Đông"}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>[{"title":"Căn hộ kiểm thử hệ thống tự động","propertyType":"Apartment","listingType":"Sale","price":3500000000,"areaSize":85,"areaUnit":"Sq M","bedrooms":2,"bathrooms":2,"locationId":1,"address":"100 Nguyễn Huệ, Phường Bến Nghé, TP. Hồ Chí Minh","ownerName":"Nguyễn Văn A","ownerPhone":"0912345678","assignedAgent":"admin","isFeatured":1,"id":21,"createdBy":"admin","created":"2026-08-21T14:39:15.248Z","updated":"2026-08-21T14:39:19.155Z","status":"Draft","viewsCount":0,"publishedAt":null,"referenceCode":"RS-LOC-1021","slug":"c-n-h-ki-m-th-h-th-ng-t-ng-21","deleted":1,"deletedAt":"2026-08-21T14:39:19.155Z","deletedBy":"admin"}]</t>
+          <t>[{"referenceCode":"RS-LAH-1012","title":"8 Marla House Bahria Sector C","slug":"8-marla-house-bahria-sector-c-12","description":"Listing being prepared — photos and owner documents pending. Not yet on the public portal.","propertyType":"House","listingType":"Sale","status":"Draft","price":31000000,"rentFrequency":"","areaSize":8,"areaUnit":"Marla","bedrooms":4,"bathrooms":4,"locationId":13,"address":"Sector C","latitude":31.3702,"longitude":74.1855,"ownerName":"Owner 12","ownerPhone":"03005000012","assignedAgent":"agent3","isFeatured":0,"viewsCount":0,"publishedAt":null,"images":[{"url":"https://picsum.photos/seed/re12a/800/500","isPrimary":1,"sortOrder":0},{"url":"https://picsum.photos/seed/re12b/800/500","isPrimary":0,"sortOrder":1},{"url":"https://picsum.photos/seed/re12c/800/500","isPrimary":0,"sortOrder":2}],"amenityIds":[1,2],"createdBy":"agent3","created":"2026-08-04T11:09:23.919Z","id":12,"updated":"2026-08-05T11:09:23.965Z"}]</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63000011444092" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -1696,7 +1715,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 5","phone":"03001000005","email":"lead5@demo.com","source":"Referral","interestType":"Buy","propertyId":3,"preferredLocationId":13,"budgetMin":7050000000,"budgetMax":8460000000,"message":"Referred by an existing client.","status":"Won","lostReason":"","assignedAgent":"agent1","createdBy":"manager1","created":"2026-07-24T11:09:26.448Z","id":5,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 5","phone":"03001000005","email":"lead5@demo.com","source":"Referral","interestType":"Buy","propertyId":3,"preferredLocationId":13,"budgetMin":75000000,"budgetMax":90000000,"message":"Referred by an existing client.","status":"Won","lostReason":"","assignedAgent":"agent1","createdBy":"manager1","created":"2026-07-24T11:09:26.448Z","id":5,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1727,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 1","phone":"03001000001","email":"lead1@demo.com","source":"Website","interestType":"Buy","propertyId":1,"preferredLocationId":11,"budgetMin":3760000000,"budgetMax":4700000000,"message":"Interested in the Phase 5 house — is the price negotiable?","status":"Negotiating","lostReason":"","assignedAgent":"agent1","createdBy":"","created":"2026-07-26T11:09:26.448Z","offers":[{"id":1,"date":"2026-08-01T11:09:26.448Z","amount":3948000000,"by":"Buyer","status":"Countered","notes":"Opening offer after first viewing","addedBy":"agent1"},{"id":2,"date":"2026-08-03T11:09:26.448Z","amount":4089000000,"by":"Seller","status":"Open","notes":"Owner counter — final offer","addedBy":"agent1"}],"id":1,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 1","phone":"03001000001","email":"lead1@demo.com","source":"Website","interestType":"Buy","propertyId":1,"preferredLocationId":11,"budgetMin":40000000,"budgetMax":50000000,"message":"Interested in the Phase 5 house — is the price negotiable?","status":"Negotiating","lostReason":"","assignedAgent":"agent1","createdBy":"","created":"2026-07-26T11:09:26.448Z","offers":[{"id":1,"date":"2026-08-01T11:09:26.448Z","amount":42000000,"by":"Buyer","status":"Countered","notes":"Opening offer after first viewing","addedBy":"agent1"},{"id":2,"date":"2026-08-03T11:09:26.448Z","amount":43500000,"by":"Seller","status":"Open","notes":"Owner counter — final offer","addedBy":"agent1"}],"id":1,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1739,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 6","phone":"03001000006","email":"","source":"Website","interestType":"Rent","propertyId":6,"preferredLocationId":15,"budgetMin":11280000,"budgetMax":15040000,"message":"Sea view apartment enquiry.","status":"Lost","lostReason":"Budget too low — rented a smaller unit elsewhere","assignedAgent":"agent2","createdBy":"","created":"2026-07-27T11:09:26.448Z","id":6,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 6","phone":"03001000006","email":"","source":"Website","interestType":"Rent","propertyId":6,"preferredLocationId":15,"budgetMin":120000,"budgetMax":160000,"message":"Sea view apartment enquiry.","status":"Lost","lostReason":"Budget too low — rented a smaller unit elsewhere","assignedAgent":"agent3","createdBy":"","created":"2026-07-27T11:09:26.448Z","id":6,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1751,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 2","phone":"03001000002","email":"lead2@demo.com","source":"WhatsApp","interestType":"Rent","propertyId":4,"preferredLocationId":6,"budgetMin":9400000,"budgetMax":13160000,"message":"Looking for a 2-bed near Main Market.","status":"Viewing Scheduled","lostReason":"","assignedAgent":"agent2","createdBy":"manager1","created":"2026-07-30T11:09:26.448Z","id":2,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 18","phone":"03001000018","email":"","source":"Website","interestType":"Rent","propertyId":14,"preferredLocationId":18,"budgetMin":6580000,"budgetMax":8460000,"message":"","status":"Lost","lostReason":"Chose a unit in another block","assignedAgent":"agent2","createdBy":"","created":"2026-07-30T11:09:26.448Z","id":18,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 2","phone":"03001000002","email":"lead2@demo.com","source":"WhatsApp","interestType":"Rent","propertyId":4,"preferredLocationId":6,"budgetMin":100000,"budgetMax":140000,"message":"Looking for a 2-bed near Main Market.","status":"Viewing Scheduled","lostReason":"","assignedAgent":"agent3","createdBy":"manager1","created":"2026-07-30T11:09:26.448Z","id":2,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 18","phone":"03001000018","email":"","source":"Website","interestType":"Rent","propertyId":14,"preferredLocationId":18,"budgetMin":70000,"budgetMax":90000,"message":"","status":"Lost","lostReason":"Chose a unit in another block","assignedAgent":"agent2","createdBy":"","created":"2026-07-30T11:09:26.448Z","id":18,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1763,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 3","phone":"03001000003","email":"","source":"Facebook","interestType":"Buy","propertyId":5,"preferredLocationId":14,"budgetMin":7520000000,"budgetMax":9400000000,"message":"Saw the Phase 8 bungalow ad.","status":"Qualified","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-07-31T11:09:26.448Z","id":3,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 3","phone":"03001000003","email":"","source":"Facebook","interestType":"Buy","propertyId":5,"preferredLocationId":14,"budgetMin":80000000,"budgetMax":100000000,"message":"Saw the Phase 8 bungalow ad.","status":"Qualified","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-07-31T11:09:26.448Z","id":3,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1775,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 4","phone":"03001000004","email":"lead4@demo.com","source":"Phone Call","interestType":"Buy","propertyId":2,"preferredLocationId":12,"budgetMin":2350000000,"budgetMax":2820000000,"message":"","status":"Contacted","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-01T11:09:26.448Z","id":4,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 15","phone":"03001000015","email":"lead15@demo.com","source":"Website","interestType":"Buy","propertyId":18,"preferredLocationId":14,"budgetMin":5170000000,"budgetMax":5828000000,"message":"Liked the corner house listing.","status":"Negotiating","lostReason":"","assignedAgent":"agent2","createdBy":"","created":"2026-08-01T11:09:26.448Z","offers":[{"id":1,"date":"2026-08-04T11:09:26.448Z","amount":5452000000,"by":"Buyer","status":"Open","notes":"Offer after the second visit","addedBy":"agent2"}],"id":15,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 4","phone":"03001000004","email":"lead4@demo.com","source":"Phone Call","interestType":"Buy","propertyId":2,"preferredLocationId":12,"budgetMin":25000000,"budgetMax":30000000,"message":"","status":"Contacted","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-01T11:09:26.448Z","id":4,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 15","phone":"03001000015","email":"lead15@demo.com","source":"Website","interestType":"Buy","propertyId":18,"preferredLocationId":14,"budgetMin":55000000,"budgetMax":62000000,"message":"Liked the corner house listing.","status":"Negotiating","lostReason":"","assignedAgent":"agent2","createdBy":"","created":"2026-08-01T11:09:26.448Z","offers":[{"id":1,"date":"2026-08-04T11:09:26.448Z","amount":58000000,"by":"Buyer","status":"Open","notes":"Offer after the second visit","addedBy":"agent2"}],"id":15,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1787,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 7","phone":"03001000007","email":"lead7@demo.com","source":"Referral","interestType":"Sell","propertyId":null,"preferredLocationId":4,"budgetMin":null,"budgetMax":null,"message":"Wants to list a 1 kanal house in DHA.","status":"Contacted","lostReason":"","assignedAgent":"agent1","createdBy":"agent1","created":"2026-08-02T11:09:26.448Z","id":7,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 13","phone":"03001000013","email":"lead13@demo.com","source":"Facebook","interestType":"Buy","propertyId":15,"preferredLocationId":20,"budgetMin":940000000,"budgetMax":1222000000,"message":"Investor — wants possession-ready plots only.","status":"Qualified","lostReason":"","assignedAgent":"agent2","createdBy":"agent3","created":"2026-08-02T11:09:26.448Z","id":13,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 19","phone":"03001000019","email":"lead19@demo.com","source":"Referral","interestType":"Buy","propertyId":2,"preferredLocationId":12,"budgetMin":2350000000,"budgetMax":2820000000,"message":"Referred by a past buyer.","status":"Qualified","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-02T11:09:26.448Z","id":19,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 7","phone":"03001000007","email":"lead7@demo.com","source":"Referral","interestType":"Sell","propertyId":null,"preferredLocationId":4,"budgetMin":null,"budgetMax":null,"message":"Wants to list a 1 kanal house in DHA.","status":"Contacted","lostReason":"","assignedAgent":"agent1","createdBy":"agent1","created":"2026-08-02T11:09:26.448Z","id":7,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 13","phone":"03001000013","email":"lead13@demo.com","source":"Facebook","interestType":"Buy","propertyId":15,"preferredLocationId":20,"budgetMin":10000000,"budgetMax":13000000,"message":"Investor — wants possession-ready plots only.","status":"Qualified","lostReason":"","assignedAgent":"agent3","createdBy":"agent3","created":"2026-08-02T11:09:26.448Z","id":13,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 19","phone":"03001000019","email":"lead19@demo.com","source":"Referral","interestType":"Buy","propertyId":2,"preferredLocationId":12,"budgetMin":25000000,"budgetMax":30000000,"message":"Referred by a past buyer.","status":"Qualified","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-02T11:09:26.448Z","id":19,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1799,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 10","phone":"03001000010","email":"lead10@demo.com","source":"Walk-in","interestType":"Buy","propertyId":null,"preferredLocationId":11,"budgetMin":3290000000,"budgetMax":4512000000,"message":"Walked into the Phase 5 office.","status":"New","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-03T11:09:26.448Z","id":10,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 12","phone":"03001000012","email":"","source":"WhatsApp","interestType":"Rent","propertyId":14,"preferredLocationId":18,"budgetMin":7520000,"budgetMax":9400000,"message":"Needs a 2-bed close to the park.","status":"Contacted","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-03T11:09:26.448Z","id":12,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 14","phone":"03001000014","email":"","source":"Referral","interestType":"Rent","propertyId":16,"preferredLocationId":6,"budgetMin":23500000,"budgetMax":28200000,"message":"Software house looking for an office floor.","status":"Viewing Scheduled","lostReason":"","assignedAgent":"agent2","createdBy":"manager1","created":"2026-08-03T11:09:26.448Z","id":14,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 17","phone":"03001000017","email":"","source":"Phone Call","interestType":"Buy","propertyId":20,"preferredLocationId":10,"budgetMin":11280000000,"budgetMax":14100000000,"message":"Farm house for family events.","status":"Contacted","lostReason":"","assignedAgent":"agent2","createdBy":"agent3","created":"2026-08-03T11:09:26.448Z","id":17,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 10","phone":"03001000010","email":"lead10@demo.com","source":"Walk-in","interestType":"Buy","propertyId":null,"preferredLocationId":11,"budgetMin":35000000,"budgetMax":48000000,"message":"Walked into the Phase 5 office.","status":"New","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-03T11:09:26.448Z","id":10,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 12","phone":"03001000012","email":"","source":"WhatsApp","interestType":"Rent","propertyId":14,"preferredLocationId":18,"budgetMin":80000,"budgetMax":100000,"message":"Needs a 2-bed close to the park.","status":"Contacted","lostReason":"","assignedAgent":"agent2","createdBy":"agent2","created":"2026-08-03T11:09:26.448Z","id":12,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 14","phone":"03001000014","email":"","source":"Referral","interestType":"Rent","propertyId":16,"preferredLocationId":6,"budgetMin":250000,"budgetMax":300000,"message":"Software house looking for an office floor.","status":"Viewing Scheduled","lostReason":"","assignedAgent":"agent2","createdBy":"manager1","created":"2026-08-03T11:09:26.448Z","id":14,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 17","phone":"03001000017","email":"","source":"Phone Call","interestType":"Buy","propertyId":20,"preferredLocationId":10,"budgetMin":120000000,"budgetMax":150000000,"message":"Farm house for family events.","status":"Contacted","lostReason":"","assignedAgent":"agent3","createdBy":"agent3","created":"2026-08-03T11:09:26.448Z","id":17,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1811,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 8","phone":"03001000008","email":"lead8@demo.com","source":"Website","interestType":"Buy","propertyId":8,"preferredLocationId":10,"budgetMin":846000000,"budgetMax":1034000000,"message":"Is the Bahria Enclave plot still available?","status":"New","lostReason":"","assignedAgent":"","createdBy":"","created":"2026-08-04T11:09:26.448Z","id":8,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 11","phone":"03001000011","email":"lead11@demo.com","source":"Website","interestType":"Buy","propertyId":13,"preferredLocationId":12,"budgetMin":2820000000,"budgetMax":3384000000,"message":"Asked for a video tour of the Phase 6 house.","status":"New","lostReason":"","assignedAgent":"","createdBy":"","created":"2026-08-04T11:09:26.448Z","id":11,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 16","phone":"03001000016","email":"","source":"Walk-in","interestType":"Sell","propertyId":null,"preferredLocationId":4,"budgetMin":null,"budgetMax":null,"message":"Wants to list a 10 marla house in DHA.","status":"New","lostReason":"","assignedAgent":"agent1","createdBy":"agent1","created":"2026-08-04T11:09:26.448Z","id":16,"updated":"2026-08-05T11:09:26.509Z"}]</t>
+          <t>[{"fullName":"Lead 8","phone":"03001000008","email":"lead8@demo.com","source":"Website","interestType":"Buy","propertyId":8,"preferredLocationId":10,"budgetMin":9000000,"budgetMax":11000000,"message":"Is the Bahria Enclave plot still available?","status":"New","lostReason":"","assignedAgent":"admin","createdBy":"","created":"2026-08-04T11:09:26.448Z","id":8,"updated":"2026-08-21T15:57:27.007Z"},{"fullName":"Lead 11","phone":"03001000011","email":"lead11@demo.com","source":"Website","interestType":"Buy","propertyId":13,"preferredLocationId":12,"budgetMin":30000000,"budgetMax":36000000,"message":"Asked for a video tour of the Phase 6 house.","status":"New","lostReason":"","assignedAgent":"admin","createdBy":"","created":"2026-08-04T11:09:26.448Z","id":11,"updated":"2026-08-21T15:57:15.380Z"},{"fullName":"Lead 16","phone":"03001000016","email":"","source":"Walk-in","interestType":"Sell","propertyId":null,"preferredLocationId":4,"budgetMin":null,"budgetMax":null,"message":"Wants to list a 10 marla house in DHA.","status":"New","lostReason":"","assignedAgent":"agent1","createdBy":"agent1","created":"2026-08-04T11:09:26.448Z","id":16,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1804,19 +1823,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[{"fullName":"Lead 9","phone":"03001000009","email":"","source":"Website","interestType":"Rent","propertyId":9,"preferredLocationId":6,"budgetMin":23500000,"budgetMax":37600000,"message":"Need a shop for a mobile accessories brand.","status":"New","lostReason":"","assignedAgent":"","createdBy":"","created":"2026-08-05T08:09:26.448Z","id":9,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 20","phone":"03001000020","email":"","source":"Website","interestType":"Rent Out","propertyId":null,"preferredLocationId":6,"budgetMin":null,"budgetMax":null,"message":"Wants to rent out an office floor in Gulberg.","status":"New","lostReason":"","assignedAgent":"","createdBy":"","created":"2026-08-05T07:09:26.448Z","id":20,"updated":"2026-08-05T11:09:26.509Z"}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>[{"fullName":"Khách hàng Test Tự Động","phone":"0988776655","email":"testlead@demo.com","source":"Website","priority":"Hot","status":"New","propertyId":21,"assignedAgent":"admin","budgetMin":3000000000,"budgetMax":4000000000,"id":21,"createdBy":"admin","created":"2026-08-21T14:39:16.207Z","updated":"2026-08-21T14:39:22.302Z","deleted":1,"deletedAt":"2026-08-21T14:39:22.302Z","deletedBy":"admin"}]</t>
+          <t>[{"fullName":"Lead 9","phone":"03001000009","email":"","source":"Website","interestType":"Rent","propertyId":9,"preferredLocationId":6,"budgetMin":250000,"budgetMax":400000,"message":"Need a shop for a mobile accessories brand.","status":"New","lostReason":"","assignedAgent":"","createdBy":"","created":"2026-08-05T08:09:26.448Z","id":9,"updated":"2026-08-05T11:09:26.509Z"},{"fullName":"Lead 20","phone":"03001000020","email":"","source":"Website","interestType":"Rent Out","propertyId":null,"preferredLocationId":6,"budgetMin":null,"budgetMax":null,"message":"Wants to rent out an office floor in Gulberg.","status":"New","lostReason":"","assignedAgent":"","createdBy":"","created":"2026-08-05T07:09:26.448Z","id":20,"updated":"2026-08-05T11:09:26.509Z"}]</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63000011444092" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -1866,7 +1873,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[{"leadId":6,"assignedAgent":"agent2","type":"Call","notes":"Final call — went with a cheaper unit","dueAt":null,"status":"Completed","completedAt":"2026-07-28T11:09:29.015Z","reminderSent":0,"createdBy":"agent3","created":"2026-07-28T11:09:29.015Z","id":6,"updated":"2026-08-05T11:09:29.064Z"}]</t>
+          <t>[{"leadId":6,"assignedAgent":"agent3","type":"Call","notes":"Final call — went with a cheaper unit","dueAt":null,"status":"Completed","completedAt":"2026-07-28T11:09:29.015Z","reminderSent":0,"createdBy":"agent3","created":"2026-07-28T11:09:29.015Z","id":6,"updated":"2026-08-05T11:09:29.064Z"}]</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1909,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[{"leadId":2,"assignedAgent":"agent2","type":"WhatsApp","notes":"Share viewing directions and parking info","dueAt":"2026-08-05T13:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:29.015Z","id":2,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":3,"assignedAgent":"agent2","type":"Call","notes":"Qualification follow-through — financing?","dueAt":"2026-08-06T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-03T11:09:29.015Z","id":3,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":10,"assignedAgent":"agent2","type":"Call","notes":"First call after walk-in visit","dueAt":"2026-08-04T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-03T11:09:29.015Z","id":8,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":13,"assignedAgent":"agent2","type":"Call","notes":"Confirm plot size preference before visit","dueAt":"2026-08-06T13:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:29.015Z","id":13,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":15,"assignedAgent":"agent2","type":"Call","notes":"Chase the counter offer","dueAt":"2026-08-04T14:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-03T11:09:29.015Z","id":15,"updated":"2026-08-05T11:09:29.064Z"}]</t>
+          <t>[{"leadId":2,"assignedAgent":"agent3","type":"WhatsApp","notes":"Share viewing directions and parking info","dueAt":"2026-08-05T13:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:29.015Z","id":2,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":3,"assignedAgent":"agent2","type":"Call","notes":"Qualification follow-through — financing?","dueAt":"2026-08-06T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-03T11:09:29.015Z","id":3,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":10,"assignedAgent":"agent2","type":"Call","notes":"First call after walk-in visit","dueAt":"2026-08-04T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-03T11:09:29.015Z","id":8,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":13,"assignedAgent":"agent3","type":"Call","notes":"Confirm plot size preference before visit","dueAt":"2026-08-06T13:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:29.015Z","id":13,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":15,"assignedAgent":"agent2","type":"Call","notes":"Chase the counter offer","dueAt":"2026-08-04T14:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-03T11:09:29.015Z","id":15,"updated":"2026-08-05T11:09:29.064Z"}]</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1921,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[{"leadId":4,"assignedAgent":"agent2","type":"Email","notes":"Send Phase 6 payment plan PDF","dueAt":"2026-08-07T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:29.015Z","id":4,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":7,"assignedAgent":"agent1","type":"Meeting","notes":"Visit seller property for valuation","dueAt":"2026-08-08T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent1","created":"2026-08-04T11:09:29.015Z","id":7,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":4,"assignedAgent":"agent2","type":"Call","notes":"Confirm interest before the weekend","dueAt":"2026-08-05T15:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:29.015Z","id":10,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":12,"assignedAgent":"agent2","type":"WhatsApp","notes":"Sent Block 7 apartment photos","dueAt":null,"status":"Completed","completedAt":"2026-08-04T11:09:29.015Z","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:29.015Z","id":12,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":14,"assignedAgent":"agent2","type":"Meeting","notes":"Office floor walk-through with their CTO","dueAt":"2026-08-07T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:29.015Z","id":14,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":16,"assignedAgent":"agent1","type":"Meeting","notes":"Valuation visit for the DHA house","dueAt":"2026-08-06T11:09:29.015Z","status":"Completed","completedAt":null,"reminderSent":0,"createdBy":"agent1","created":"2026-08-04T11:09:29.015Z","id":16,"updated":"2026-08-21T10:01:30.586Z"},{"leadId":17,"assignedAgent":"agent2","type":"Email","notes":"Send farm house event-lawn photos","dueAt":"2026-08-08T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent3","created":"2026-08-04T11:09:29.015Z","id":17,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":19,"assignedAgent":"agent2","type":"Call","notes":"Arrange a Phase 6 house visit","dueAt":"2026-08-05T17:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:29.015Z","id":19,"updated":"2026-08-05T11:09:29.064Z"}]</t>
+          <t>[{"leadId":4,"assignedAgent":"agent2","type":"Email","notes":"Send Phase 6 payment plan PDF","dueAt":"2026-08-07T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:29.015Z","id":4,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":7,"assignedAgent":"agent1","type":"Meeting","notes":"Visit seller property for valuation","dueAt":"2026-08-08T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent1","created":"2026-08-04T11:09:29.015Z","id":7,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":4,"assignedAgent":"agent2","type":"Call","notes":"Confirm interest before the weekend","dueAt":"2026-08-05T15:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:29.015Z","id":10,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":12,"assignedAgent":"agent2","type":"WhatsApp","notes":"Sent Block 7 apartment photos","dueAt":null,"status":"Completed","completedAt":"2026-08-04T11:09:29.015Z","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:29.015Z","id":12,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":14,"assignedAgent":"agent2","type":"Meeting","notes":"Office floor walk-through with their CTO","dueAt":"2026-08-07T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:29.015Z","id":14,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":16,"assignedAgent":"agent1","type":"Meeting","notes":"Valuation visit for the DHA house","dueAt":"2026-08-06T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent1","created":"2026-08-04T11:09:29.015Z","id":16,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":17,"assignedAgent":"agent3","type":"Email","notes":"Send farm house event-lawn photos","dueAt":"2026-08-08T11:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent3","created":"2026-08-04T11:09:29.015Z","id":17,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":19,"assignedAgent":"agent2","type":"Call","notes":"Arrange a Phase 6 house visit","dueAt":"2026-08-05T17:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:29.015Z","id":19,"updated":"2026-08-05T11:09:29.064Z"}]</t>
         </is>
       </c>
     </row>
@@ -1927,18 +1934,6 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>[{"leadId":11,"assignedAgent":"manager1","type":"Call","notes":"First contact — assign an agent after","dueAt":"2026-08-05T14:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"manager1","created":"2026-08-05T09:09:29.015Z","id":11,"updated":"2026-08-05T11:09:29.064Z"},{"leadId":20,"assignedAgent":"manager1","type":"Call","notes":"Collect office details for the listing","dueAt":"2026-08-05T16:09:29.015Z","status":"Pending","completedAt":null,"reminderSent":0,"createdBy":"manager1","created":"2026-08-05T08:09:29.015Z","id":20,"updated":"2026-08-05T11:09:29.064Z"}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>[{"leadId":21,"type":"Call","notes":"Gọi điện xác nhận lịch xem 25/08","dueAt":"2026-08-24T15:00","id":21,"createdBy":"admin","created":"2026-08-21T14:39:18.192Z","updated":"2026-08-21T14:39:18.192Z","status":"Pending","assignedAgent":"admin"}]</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63000011444092" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -1988,7 +1983,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[{"leadId":6,"propertyId":6,"agent":"agent2","scheduledAt":"2026-07-28T11:09:30.111Z","durationMinutes":45,"status":"No Show","notes":"Did not answer calls at slot time","cancellationReason":"","reminderSent":1,"createdBy":"agent3","created":"2026-07-27T11:09:30.111Z","id":6,"updated":"2026-08-05T11:09:30.164Z"}]</t>
+          <t>[{"leadId":6,"propertyId":6,"agent":"agent3","scheduledAt":"2026-07-28T11:09:30.111Z","durationMinutes":45,"status":"No Show","notes":"Did not answer calls at slot time","cancellationReason":"","reminderSent":1,"createdBy":"agent3","created":"2026-07-27T11:09:30.111Z","id":6,"updated":"2026-08-05T11:09:30.164Z"}]</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2031,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[{"leadId":13,"propertyId":8,"agent":"agent2","scheduledAt":"2026-08-03T11:09:30.111Z","durationMinutes":30,"status":"Completed","notes":"","cancellationReason":"","reminderSent":1,"createdBy":"agent3","created":"2026-08-02T11:09:30.111Z","interestLevel":"Warm","feedback":"Wants a bigger plot on the same road","id":17,"updated":"2026-08-05T11:09:30.164Z"}]</t>
+          <t>[{"leadId":13,"propertyId":8,"agent":"agent3","scheduledAt":"2026-08-03T11:09:30.111Z","durationMinutes":30,"status":"Completed","notes":"","cancellationReason":"","reminderSent":1,"createdBy":"agent3","created":"2026-08-02T11:09:30.111Z","interestLevel":"Warm","feedback":"Wants a bigger plot on the same road","id":17,"updated":"2026-08-05T11:09:30.164Z"}]</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2043,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[{"leadId":2,"propertyId":4,"agent":"agent2","scheduledAt":"2026-08-05T14:09:30.110Z","durationMinutes":45,"status":"Confirmed","notes":"Client will bring spouse","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:30.111Z","id":1,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":13,"propertyId":15,"agent":"agent2","scheduledAt":"2026-08-07T13:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"Meet at the society gate","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:30.111Z","id":11,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":16,"propertyId":1,"agent":"agent1","scheduledAt":"2026-08-04T13:09:30.111Z","durationMinutes":30,"status":"Cancelled","notes":"","cancellationReason":"Seller rescheduled the valuation","reminderSent":1,"createdBy":"agent1","created":"2026-08-03T11:09:30.111Z","id":20,"updated":"2026-08-05T11:09:30.164Z"}]</t>
+          <t>[{"leadId":2,"propertyId":4,"agent":"agent3","scheduledAt":"2026-08-05T14:09:30.110Z","durationMinutes":45,"status":"Confirmed","notes":"Client will bring spouse","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:30.111Z","id":1,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":13,"propertyId":15,"agent":"agent3","scheduledAt":"2026-08-07T13:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"Meet at the society gate","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-03T11:09:30.111Z","id":11,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":16,"propertyId":1,"agent":"agent1","scheduledAt":"2026-08-04T13:09:30.111Z","durationMinutes":30,"status":"Cancelled","notes":"","cancellationReason":"Seller rescheduled the valuation","reminderSent":1,"createdBy":"agent1","created":"2026-08-03T11:09:30.111Z","id":20,"updated":"2026-08-05T11:09:30.164Z"}]</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2055,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[{"leadId":1,"propertyId":1,"agent":"agent1","scheduledAt":"2026-08-06T13:09:30.111Z","durationMinutes":60,"status":"Scheduled","notes":"Second visit — measurements","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:30.111Z","id":2,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":3,"propertyId":5,"agent":"agent2","scheduledAt":"2026-08-07T11:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":3,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":10,"propertyId":2,"agent":"agent2","scheduledAt":"2026-08-09T11:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"First viewing","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":4,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":12,"propertyId":14,"agent":"agent2","scheduledAt":"2026-08-06T17:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":10,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":14,"propertyId":16,"agent":"agent2","scheduledAt":"2026-08-07T16:09:30.111Z","durationMinutes":60,"status":"Confirmed","notes":"CTO joining the walk-through","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:30.111Z","id":12,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":17,"propertyId":20,"agent":"agent2","scheduledAt":"2026-08-08T15:09:30.111Z","durationMinutes":60,"status":"Scheduled","notes":"Family visit — weekend slot","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-04T11:09:30.111Z","id":14,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":19,"propertyId":2,"agent":"agent2","scheduledAt":"2026-08-09T13:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":15,"updated":"2026-08-05T11:09:30.164Z"}]</t>
+          <t>[{"leadId":1,"propertyId":1,"agent":"agent1","scheduledAt":"2026-08-06T13:09:30.111Z","durationMinutes":60,"status":"Scheduled","notes":"Second visit — measurements","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:30.111Z","id":2,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":3,"propertyId":5,"agent":"agent2","scheduledAt":"2026-08-07T11:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":3,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":10,"propertyId":2,"agent":"agent2","scheduledAt":"2026-08-09T11:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"First viewing","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":4,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":12,"propertyId":14,"agent":"agent2","scheduledAt":"2026-08-06T17:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":10,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":14,"propertyId":16,"agent":"agent2","scheduledAt":"2026-08-07T16:09:30.111Z","durationMinutes":60,"status":"Confirmed","notes":"CTO joining the walk-through","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-04T11:09:30.111Z","id":12,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":17,"propertyId":20,"agent":"agent3","scheduledAt":"2026-08-08T15:09:30.111Z","durationMinutes":60,"status":"Scheduled","notes":"Family visit — weekend slot","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-04T11:09:30.111Z","id":14,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":19,"propertyId":2,"agent":"agent2","scheduledAt":"2026-08-09T13:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"","cancellationReason":"","reminderSent":0,"createdBy":"agent2","created":"2026-08-04T11:09:30.111Z","id":15,"updated":"2026-08-05T11:09:30.164Z"}]</t>
         </is>
       </c>
     </row>
@@ -2072,19 +2067,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[{"leadId":2,"propertyId":6,"agent":"agent2","scheduledAt":"2026-08-06T16:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"Backup option if Gulberg falls through","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-05T09:09:30.111Z","id":8,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":11,"propertyId":13,"agent":"manager1","scheduledAt":"2026-08-06T14:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"Unassigned lead — manager covering","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-05T10:09:30.111Z","id":9,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":20,"propertyId":16,"agent":"manager1","scheduledAt":"2026-08-06T19:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"Owner-side visit for the new listing","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-05T08:09:30.111Z","id":18,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":17,"propertyId":5,"agent":"agent2","scheduledAt":"2026-08-10T14:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"Backup option — bungalow","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-05T07:09:30.111Z","id":19,"updated":"2026-08-05T11:09:30.164Z"}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>[{"leadId":"20","propertyId":"12","agent":"admin","scheduledAt":"2026-07-31T12:52","durationMinutes":"30","notes":"","id":21,"createdBy":"admin","created":"2026-08-21T05:50:24.200Z","updated":"2026-08-21T05:50:24.200Z","status":"Scheduled"},{"leadId":21,"propertyId":21,"scheduledAt":"2026-08-25T09:00","type":"Viewing","notes":"Khách muốn xem thực tế hướng ban công","agent":"admin","id":22,"createdBy":"admin","created":"2026-08-21T14:39:17.172Z","updated":"2026-08-21T14:39:17.172Z","status":"Scheduled"}]</t>
+          <t>[{"leadId":2,"propertyId":6,"agent":"agent3","scheduledAt":"2026-08-06T16:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"Backup option if Gulberg falls through","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-05T09:09:30.111Z","id":8,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":11,"propertyId":13,"agent":"manager1","scheduledAt":"2026-08-06T14:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"Unassigned lead — manager covering","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-05T10:09:30.111Z","id":9,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":20,"propertyId":16,"agent":"manager1","scheduledAt":"2026-08-06T19:09:30.111Z","durationMinutes":30,"status":"Scheduled","notes":"Owner-side visit for the new listing","cancellationReason":"","reminderSent":0,"createdBy":"manager1","created":"2026-08-05T08:09:30.111Z","id":18,"updated":"2026-08-05T11:09:30.164Z"},{"leadId":17,"propertyId":5,"agent":"agent3","scheduledAt":"2026-08-10T14:09:30.111Z","durationMinutes":45,"status":"Scheduled","notes":"Backup option — bungalow","cancellationReason":"","reminderSent":0,"createdBy":"agent3","created":"2026-08-05T07:09:30.111Z","id":19,"updated":"2026-08-05T11:09:30.164Z"}]</t>
         </is>
       </c>
     </row>

</xml_diff>